<commit_message>
chore(tracker): actualizacion diaria de vacantes 2026-10-04
</commit_message>
<xml_diff>
--- a/output/profile_6_auxiliar_administrativo_tracker.xlsx
+++ b/output/profile_6_auxiliar_administrativo_tracker.xlsx
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K167"/>
+  <dimension ref="A1:K168"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3114,26 +3114,26 @@
     <row r="57" ht="22" customHeight="1">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>d7b10cded83b71f2</t>
+          <t>aa44c6d913e4d552</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 16:07</t>
+          <t>2026-10-04 15:51</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>Analista junior de facturación y telecomunicaciones</t>
+          <t>Auxiliar de facturación - puente aranda- 1625881713-123</t>
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>TP COLOMBIA</t>
+          <t>AGENCIA DE EMPLEO Y FOMENTO EMPRESARIAL COMPENSAR</t>
         </is>
       </c>
       <c r="E57" s="4" t="n">
-        <v>0.7</v>
+        <v>0.73</v>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
@@ -3141,13 +3141,13 @@
         </is>
       </c>
       <c r="G57" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-junior-de-facturacion-y-telecomunicaciones-1886758607", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-facturacion-puente-aranda-1625881713123-1886769348", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H57" s="6" t="inlineStr"/>
       <c r="I57" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 70/100 - Alta Afinidad] Alta coincidencia técnica en Herramientas Ofimáticas, Excel y Soporte Contable / Facturación. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 73/100 - Alta Afinidad] Alta coincidencia técnica en Herramientas Ofimáticas, Excel y Soporte Contable / Facturación. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J57" s="2" t="inlineStr">
@@ -3160,7 +3160,7 @@
     <row r="58" ht="22" customHeight="1">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>7c8e4b63802fbfdd</t>
+          <t>d7b10cded83b71f2</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -3170,16 +3170,16 @@
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>Analista de facturacion - mocoa</t>
+          <t>Analista junior de facturación y telecomunicaciones</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>Clínica Medilaser S.A.S</t>
-        </is>
-      </c>
-      <c r="E58" s="7" t="n">
-        <v>0.68</v>
+          <t>TP COLOMBIA</t>
+        </is>
+      </c>
+      <c r="E58" s="4" t="n">
+        <v>0.7</v>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
@@ -3187,13 +3187,13 @@
         </is>
       </c>
       <c r="G58" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-facturacion-mocoa-1886758704", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-junior-de-facturacion-y-telecomunicaciones-1886758607", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H58" s="6" t="inlineStr"/>
       <c r="I58" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 68/100 - Afinidad Moderada] Alta coincidencia técnica en Herramientas Ofimáticas, Excel y Soporte Contable / Facturación. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 70/100 - Alta Afinidad] Alta coincidencia técnica en Herramientas Ofimáticas, Excel y Soporte Contable / Facturación. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J58" s="2" t="inlineStr">
@@ -3206,7 +3206,7 @@
     <row r="59" ht="22" customHeight="1">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>6a1a399dbe055821</t>
+          <t>7c8e4b63802fbfdd</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
@@ -3216,12 +3216,12 @@
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>Analista de facturación</t>
+          <t>Analista de facturacion - mocoa</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>CONTINAUTOS S.A.</t>
+          <t>Clínica Medilaser S.A.S</t>
         </is>
       </c>
       <c r="E59" s="7" t="n">
@@ -3233,7 +3233,7 @@
         </is>
       </c>
       <c r="G59" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-facturacion-1886758032", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-facturacion-mocoa-1886758704", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H59" s="6" t="inlineStr"/>
@@ -3252,7 +3252,7 @@
     <row r="60" ht="22" customHeight="1">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>8d104e6e0596782f</t>
+          <t>6a1a399dbe055821</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
@@ -3262,12 +3262,12 @@
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>Analista de facturación - zipaquira</t>
+          <t>Analista de facturación</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>CONTINAUTOS S.A.</t>
         </is>
       </c>
       <c r="E60" s="7" t="n">
@@ -3279,7 +3279,7 @@
         </is>
       </c>
       <c r="G60" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-facturacion-zipaquira-1886769380", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-facturacion-1886758032", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H60" s="6" t="inlineStr"/>
@@ -3298,7 +3298,7 @@
     <row r="61" ht="22" customHeight="1">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>30c981b787bd9e84</t>
+          <t>8d104e6e0596782f</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
@@ -3308,12 +3308,12 @@
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>Analista de facturación</t>
+          <t>Analista de facturación - zipaquira</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>IMPULSO TEMPORAL SAS</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E61" s="7" t="n">
@@ -3325,7 +3325,7 @@
         </is>
       </c>
       <c r="G61" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-facturacion-1886751641", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-facturacion-zipaquira-1886769380", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H61" s="6" t="inlineStr"/>
@@ -3344,7 +3344,7 @@
     <row r="62" ht="22" customHeight="1">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>6ba85335e71be4cc</t>
+          <t>30c981b787bd9e84</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -3354,12 +3354,12 @@
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>Analista de Facturacion</t>
+          <t>Analista de facturación</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>Experian Spanish Latam</t>
+          <t>IMPULSO TEMPORAL SAS</t>
         </is>
       </c>
       <c r="E62" s="7" t="n">
@@ -3371,7 +3371,7 @@
         </is>
       </c>
       <c r="G62" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/analista-de-facturacion-at-experian-spanish-latam-4462035775", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-facturacion-1886751641", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H62" s="6" t="inlineStr"/>
@@ -3390,7 +3390,7 @@
     <row r="63" ht="22" customHeight="1">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>0ba2c0ed565928ee</t>
+          <t>6ba85335e71be4cc</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
@@ -3400,12 +3400,12 @@
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>Analista de facturación y gasto</t>
+          <t>Analista de Facturacion</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>AXA Partners</t>
+          <t>Experian Spanish Latam</t>
         </is>
       </c>
       <c r="E63" s="7" t="n">
@@ -3417,7 +3417,7 @@
         </is>
       </c>
       <c r="G63" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/analista-de-facturaci%C3%B3n-y-gasto-at-axa-partners-4468296274", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/analista-de-facturacion-at-experian-spanish-latam-4462035775", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H63" s="6" t="inlineStr"/>
@@ -3436,7 +3436,7 @@
     <row r="64" ht="22" customHeight="1">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2adbc58cb85c19c7</t>
+          <t>0ba2c0ed565928ee</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -3446,12 +3446,12 @@
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>Analista de Facturación de servicios</t>
+          <t>Analista de facturación y gasto</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
-          <t>Américas BPS</t>
+          <t>AXA Partners</t>
         </is>
       </c>
       <c r="E64" s="7" t="n">
@@ -3463,7 +3463,7 @@
         </is>
       </c>
       <c r="G64" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/analista-de-facturaci%C3%B3n-de-servicios-at-am%C3%A9ricas-bps-4464891719", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/analista-de-facturaci%C3%B3n-y-gasto-at-axa-partners-4468296274", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H64" s="6" t="inlineStr"/>
@@ -3482,22 +3482,22 @@
     <row r="65" ht="22" customHeight="1">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>a831855f10d17417</t>
+          <t>2adbc58cb85c19c7</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 15:56</t>
+          <t>2026-09-24 16:07</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>Analista de facturación</t>
+          <t>Analista de Facturación de servicios</t>
         </is>
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Américas BPS</t>
         </is>
       </c>
       <c r="E65" s="7" t="n">
@@ -3509,7 +3509,7 @@
         </is>
       </c>
       <c r="G65" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-facturacion-1886756696", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/analista-de-facturaci%C3%B3n-de-servicios-at-am%C3%A9ricas-bps-4464891719", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H65" s="6" t="inlineStr"/>
@@ -3528,7 +3528,7 @@
     <row r="66" ht="22" customHeight="1">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>d59df408fc52566d</t>
+          <t>a831855f10d17417</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -3538,7 +3538,7 @@
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>Analista de facturación- manejo de sap -</t>
+          <t>Analista de facturación</t>
         </is>
       </c>
       <c r="D66" s="3" t="inlineStr">
@@ -3555,7 +3555,7 @@
         </is>
       </c>
       <c r="G66" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-facturacion-manejo-de-sap-1886756806", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-facturacion-1886756696", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H66" s="6" t="inlineStr"/>
@@ -3574,7 +3574,7 @@
     <row r="67" ht="22" customHeight="1">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>a1b8ba55f8922e99</t>
+          <t>d59df408fc52566d</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
@@ -3584,12 +3584,12 @@
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>Analista de cartera y facturación</t>
+          <t>Analista de facturación- manejo de sap -</t>
         </is>
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t>MENTORHUB COLOMBIA</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E67" s="7" t="n">
@@ -3601,7 +3601,7 @@
         </is>
       </c>
       <c r="G67" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-cartera-y-facturacion-1886741299", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-facturacion-manejo-de-sap-1886756806", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H67" s="6" t="inlineStr"/>
@@ -3620,22 +3620,22 @@
     <row r="68" ht="22" customHeight="1">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>62e18b4bd9d42926</t>
+          <t>a1b8ba55f8922e99</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26 15:05</t>
+          <t>2026-09-25 15:56</t>
         </is>
       </c>
       <c r="C68" s="3" t="inlineStr">
         <is>
-          <t>Analista de control operativo y facturación aduanera</t>
+          <t>Analista de cartera y facturación</t>
         </is>
       </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
-          <t>crane ww logistics</t>
+          <t>MENTORHUB COLOMBIA</t>
         </is>
       </c>
       <c r="E68" s="7" t="n">
@@ -3647,7 +3647,7 @@
         </is>
       </c>
       <c r="G68" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-control-operativo-y-facturacion-aduanera-1886771256", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-cartera-y-facturacion-1886741299", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H68" s="6" t="inlineStr"/>
@@ -3666,22 +3666,22 @@
     <row r="69" ht="22" customHeight="1">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>62ab67e660127864</t>
+          <t>62e18b4bd9d42926</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 18:38</t>
+          <t>2026-09-26 15:05</t>
         </is>
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>Analista de facturación y cartera</t>
+          <t>Analista de control operativo y facturación aduanera</t>
         </is>
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>DON MAKINON</t>
+          <t>crane ww logistics</t>
         </is>
       </c>
       <c r="E69" s="7" t="n">
@@ -3693,7 +3693,7 @@
         </is>
       </c>
       <c r="G69" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-facturacion-y-cartera-1886773105", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-control-operativo-y-facturacion-aduanera-1886771256", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H69" s="6" t="inlineStr"/>
@@ -3712,22 +3712,22 @@
     <row r="70" ht="22" customHeight="1">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>39bf6fcb2b2ffb07</t>
+          <t>62ab67e660127864</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 16:51</t>
+          <t>2026-09-28 18:38</t>
         </is>
       </c>
       <c r="C70" s="3" t="inlineStr">
         <is>
-          <t>Analista de facturación - medellín</t>
+          <t>Analista de facturación y cartera</t>
         </is>
       </c>
       <c r="D70" s="3" t="inlineStr">
         <is>
-          <t>SERVICIOS DE AUDITORIA Y CONSULTORIA DE NEGOCIOS SAS</t>
+          <t>DON MAKINON</t>
         </is>
       </c>
       <c r="E70" s="7" t="n">
@@ -3739,7 +3739,7 @@
         </is>
       </c>
       <c r="G70" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-facturacion-medellin-1886754458", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-facturacion-y-cartera-1886773105", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H70" s="6" t="inlineStr"/>
@@ -3758,26 +3758,26 @@
     <row r="71" ht="22" customHeight="1">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>8ea64e48a843110e</t>
+          <t>39bf6fcb2b2ffb07</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 16:07</t>
+          <t>2026-09-30 16:51</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar de Digitación y Validación de Información</t>
+          <t>Analista de facturación - medellín</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>Hy Cite</t>
+          <t>SERVICIOS DE AUDITORIA Y CONSULTORIA DE NEGOCIOS SAS</t>
         </is>
       </c>
       <c r="E71" s="7" t="n">
-        <v>0.66</v>
+        <v>0.68</v>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
@@ -3785,13 +3785,13 @@
         </is>
       </c>
       <c r="G71" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/auxiliar-de-digitaci%C3%B3n-y-validaci%C3%B3n-de-informaci%C3%B3n-at-hy-cite-4444163970", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-facturacion-medellin-1886754458", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H71" s="6" t="inlineStr"/>
       <c r="I71" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 66/100 - Afinidad Moderada] Alta coincidencia técnica en Gestión Administrativa, Documental y Archivo. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 68/100 - Afinidad Moderada] Alta coincidencia técnica en Herramientas Ofimáticas, Excel y Soporte Contable / Facturación. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J71" s="2" t="inlineStr">
@@ -3804,7 +3804,7 @@
     <row r="72" ht="22" customHeight="1">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>0810fb157c23918e</t>
+          <t>8ea64e48a843110e</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
@@ -3814,16 +3814,16 @@
       </c>
       <c r="C72" s="3" t="inlineStr">
         <is>
-          <t>Junior Tax Accountant / Data entry</t>
+          <t>Auxiliar de Digitación y Validación de Información</t>
         </is>
       </c>
       <c r="D72" s="3" t="inlineStr">
         <is>
-          <t>George Dimov, CPA</t>
+          <t>Hy Cite</t>
         </is>
       </c>
       <c r="E72" s="7" t="n">
-        <v>0.6</v>
+        <v>0.66</v>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
@@ -3831,13 +3831,13 @@
         </is>
       </c>
       <c r="G72" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/junior-tax-accountant-data-entry-remote-at-george-dimov-cpa-4468922588", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/auxiliar-de-digitaci%C3%B3n-y-validaci%C3%B3n-de-informaci%C3%B3n-at-hy-cite-4444163970", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H72" s="6" t="inlineStr"/>
       <c r="I72" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 60/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Auxiliar Administrativo / Asistente Virtual). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 66/100 - Afinidad Moderada] Alta coincidencia técnica en Gestión Administrativa, Documental y Archivo. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J72" s="2" t="inlineStr">
@@ -3850,7 +3850,7 @@
     <row r="73" ht="22" customHeight="1">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>b9e81da0bd12d416</t>
+          <t>0810fb157c23918e</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
@@ -3860,16 +3860,16 @@
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar administrativo</t>
+          <t>Junior Tax Accountant / Data entry</t>
         </is>
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>VR RISK</t>
+          <t>George Dimov, CPA</t>
         </is>
       </c>
       <c r="E73" s="7" t="n">
-        <v>0.58</v>
+        <v>0.6</v>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
@@ -3877,17 +3877,13 @@
         </is>
       </c>
       <c r="G73" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-administrativo-remoto-en-bogota-dc-08C32BD16679929A61373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H73" s="6" t="inlineStr">
-        <is>
-          <t>$ 2.000.000,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/junior-tax-accountant-data-entry-remote-at-george-dimov-cpa-4468922588", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H73" s="6" t="inlineStr"/>
       <c r="I73" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Auxiliar Administrativo / Asistente Virtual). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 60/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Auxiliar Administrativo / Asistente Virtual). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J73" s="2" t="inlineStr">
@@ -3900,7 +3896,7 @@
     <row r="74" ht="22" customHeight="1">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>60a767236cb83e2b</t>
+          <t>b9e81da0bd12d416</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
@@ -3910,12 +3906,12 @@
       </c>
       <c r="C74" s="3" t="inlineStr">
         <is>
-          <t>Asistente Administrativo y de Operaciones</t>
+          <t>Auxiliar administrativo</t>
         </is>
       </c>
       <c r="D74" s="3" t="inlineStr">
         <is>
-          <t>Direct Home Solutions</t>
+          <t>VR RISK</t>
         </is>
       </c>
       <c r="E74" s="7" t="n">
@@ -3927,12 +3923,12 @@
         </is>
       </c>
       <c r="G74" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-asistente-administrativo-y-de-operaciones-remoto-en-pereira-737F61DE07AA2E7F61373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-administrativo-remoto-en-bogota-dc-08C32BD16679929A61373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H74" s="6" t="inlineStr">
         <is>
-          <t>$ 2.600.000,00 (Mensual)</t>
+          <t>$ 2.000.000,00 (Mensual)</t>
         </is>
       </c>
       <c r="I74" s="3" t="inlineStr">
@@ -3950,7 +3946,7 @@
     <row r="75" ht="22" customHeight="1">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>04855c966d018926</t>
+          <t>60a767236cb83e2b</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
@@ -3960,12 +3956,12 @@
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar administrativo/a Vacante Inclusiva para personas con Discapacidad</t>
+          <t>Asistente Administrativo y de Operaciones</t>
         </is>
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>CENTRO DE EMPLEO Y TALENTO COLSUBSIDIO</t>
+          <t>Direct Home Solutions</t>
         </is>
       </c>
       <c r="E75" s="7" t="n">
@@ -3977,12 +3973,12 @@
         </is>
       </c>
       <c r="G75" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-administrativoa-vacante-inclusiva-para-personas-con-discapacidad-en-bogota-dc-F5B96991A8C617B661373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-asistente-administrativo-y-de-operaciones-remoto-en-pereira-737F61DE07AA2E7F61373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H75" s="6" t="inlineStr">
         <is>
-          <t>$ 2.000.000,00 (Mensual)</t>
+          <t>$ 2.600.000,00 (Mensual)</t>
         </is>
       </c>
       <c r="I75" s="3" t="inlineStr">
@@ -4000,7 +3996,7 @@
     <row r="76" ht="22" customHeight="1">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>a30e3afa7b66502b</t>
+          <t>04855c966d018926</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
@@ -4010,12 +4006,12 @@
       </c>
       <c r="C76" s="3" t="inlineStr">
         <is>
-          <t>auxiliar administrativo/a</t>
+          <t>Auxiliar administrativo/a Vacante Inclusiva para personas con Discapacidad</t>
         </is>
       </c>
       <c r="D76" s="3" t="inlineStr">
         <is>
-          <t>ELITE SKIN ITALY S.A.S</t>
+          <t>CENTRO DE EMPLEO Y TALENTO COLSUBSIDIO</t>
         </is>
       </c>
       <c r="E76" s="7" t="n">
@@ -4027,7 +4023,7 @@
         </is>
       </c>
       <c r="G76" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-administrativoa-virtual-remoto-con-o-sin-experiencia-en-bogota-dc-246C4633B2C1D28D61373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-administrativoa-vacante-inclusiva-para-personas-con-discapacidad-en-bogota-dc-F5B96991A8C617B661373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H76" s="6" t="inlineStr">
@@ -4050,7 +4046,7 @@
     <row r="77" ht="22" customHeight="1">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>899512a1b5af847f</t>
+          <t>a30e3afa7b66502b</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
@@ -4060,12 +4056,12 @@
       </c>
       <c r="C77" s="3" t="inlineStr">
         <is>
-          <t>auxiliar contable y administrativo</t>
+          <t>auxiliar administrativo/a</t>
         </is>
       </c>
       <c r="D77" s="3" t="inlineStr">
         <is>
-          <t>AZ LOGICA SAS</t>
+          <t>ELITE SKIN ITALY S.A.S</t>
         </is>
       </c>
       <c r="E77" s="7" t="n">
@@ -4077,7 +4073,7 @@
         </is>
       </c>
       <c r="G77" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-contable-y-administrativo-en-bogota-dc-E79FB52CC71B1AAF61373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-administrativoa-virtual-remoto-con-o-sin-experiencia-en-bogota-dc-246C4633B2C1D28D61373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H77" s="6" t="inlineStr">
@@ -4100,7 +4096,7 @@
     <row r="78" ht="22" customHeight="1">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>0048b5632ef5acf6</t>
+          <t>899512a1b5af847f</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
@@ -4110,12 +4106,12 @@
       </c>
       <c r="C78" s="3" t="inlineStr">
         <is>
-          <t>Asistente Administrativo</t>
+          <t>auxiliar contable y administrativo</t>
         </is>
       </c>
       <c r="D78" s="3" t="inlineStr">
         <is>
-          <t>Naonsoft</t>
+          <t>AZ LOGICA SAS</t>
         </is>
       </c>
       <c r="E78" s="7" t="n">
@@ -4127,12 +4123,12 @@
         </is>
       </c>
       <c r="G78" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-asistente-administrativo-en-medellin-268B37E50FB0D28461373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-contable-y-administrativo-en-bogota-dc-E79FB52CC71B1AAF61373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H78" s="6" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>$ 2.000.000,00 (Mensual)</t>
         </is>
       </c>
       <c r="I78" s="3" t="inlineStr">
@@ -4150,7 +4146,7 @@
     <row r="79" ht="22" customHeight="1">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>062ee3244ed08bb4</t>
+          <t>0048b5632ef5acf6</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
@@ -4160,12 +4156,12 @@
       </c>
       <c r="C79" s="3" t="inlineStr">
         <is>
-          <t>Asistente de Servicio al Cliente y Administrativo</t>
+          <t>Asistente Administrativo</t>
         </is>
       </c>
       <c r="D79" s="3" t="inlineStr">
         <is>
-          <t>Health and Fitness</t>
+          <t>Naonsoft</t>
         </is>
       </c>
       <c r="E79" s="7" t="n">
@@ -4177,12 +4173,12 @@
         </is>
       </c>
       <c r="G79" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-asistente-de-servicio-al-cliente-y-administrativo-ingles-nativo-requerido-ingles-nativo-requerido-en-colombia-BA7538B8C571FA9F61373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-asistente-administrativo-en-medellin-268B37E50FB0D28461373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H79" s="6" t="inlineStr">
         <is>
-          <t>$ 2.500.000,00 (Mensual)</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="I79" s="3" t="inlineStr">
@@ -4200,7 +4196,7 @@
     <row r="80" ht="22" customHeight="1">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>90d5245bdef0186a</t>
+          <t>062ee3244ed08bb4</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
@@ -4210,12 +4206,12 @@
       </c>
       <c r="C80" s="3" t="inlineStr">
         <is>
-          <t>Asistente administrativo y financiero</t>
+          <t>Asistente de Servicio al Cliente y Administrativo</t>
         </is>
       </c>
       <c r="D80" s="3" t="inlineStr">
         <is>
-          <t>SOLVO S.A.S</t>
+          <t>Health and Fitness</t>
         </is>
       </c>
       <c r="E80" s="7" t="n">
@@ -4227,12 +4223,12 @@
         </is>
       </c>
       <c r="G80" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-asistente-administrativo-y-financiero-b2-en-bogota-dc-8B5C137D8309F1F661373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-asistente-de-servicio-al-cliente-y-administrativo-ingles-nativo-requerido-ingles-nativo-requerido-en-colombia-BA7538B8C571FA9F61373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H80" s="6" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>$ 2.500.000,00 (Mensual)</t>
         </is>
       </c>
       <c r="I80" s="3" t="inlineStr">
@@ -4250,7 +4246,7 @@
     <row r="81" ht="22" customHeight="1">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>760f13e3724f6b31</t>
+          <t>90d5245bdef0186a</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
@@ -4277,7 +4273,7 @@
         </is>
       </c>
       <c r="G81" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-asistente-administrativo-y-financiero-b2-en-medellin-837774FFD1C514D261373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-asistente-administrativo-y-financiero-b2-en-bogota-dc-8B5C137D8309F1F661373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H81" s="6" t="inlineStr">
@@ -4300,7 +4296,7 @@
     <row r="82" ht="22" customHeight="1">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2d0d5c2d341e3d17</t>
+          <t>760f13e3724f6b31</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
@@ -4327,7 +4323,7 @@
         </is>
       </c>
       <c r="G82" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-asistente-administrativo-y-financiero-b2-en-barranquilla-08F31F737CD14CED61373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-asistente-administrativo-y-financiero-b2-en-medellin-837774FFD1C514D261373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H82" s="6" t="inlineStr">
@@ -4350,7 +4346,7 @@
     <row r="83" ht="22" customHeight="1">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>63592c52663ab0e0</t>
+          <t>2d0d5c2d341e3d17</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
@@ -4360,12 +4356,12 @@
       </c>
       <c r="C83" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar administrativo horario flexible remoto</t>
+          <t>Asistente administrativo y financiero</t>
         </is>
       </c>
       <c r="D83" s="3" t="inlineStr">
         <is>
-          <t>Empire Co</t>
+          <t>SOLVO S.A.S</t>
         </is>
       </c>
       <c r="E83" s="7" t="n">
@@ -4377,10 +4373,14 @@
         </is>
       </c>
       <c r="G83" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-administrativo-horario-flexible-remoto-1886769479", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H83" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-asistente-administrativo-y-financiero-b2-en-barranquilla-08F31F737CD14CED61373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H83" s="6" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
       <c r="I83" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Auxiliar Administrativo / Asistente Virtual). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -4396,7 +4396,7 @@
     <row r="84" ht="22" customHeight="1">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>729fb015086632d9</t>
+          <t>63592c52663ab0e0</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
@@ -4406,12 +4406,12 @@
       </c>
       <c r="C84" s="3" t="inlineStr">
         <is>
-          <t>Asistente de cuentas por pagar o tesoreria -remoto</t>
+          <t>Auxiliar administrativo horario flexible remoto</t>
         </is>
       </c>
       <c r="D84" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Empire Co</t>
         </is>
       </c>
       <c r="E84" s="7" t="n">
@@ -4423,7 +4423,7 @@
         </is>
       </c>
       <c r="G84" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/asistente-de-cuentas-por-pagar-o-tesoreria-remoto-1886744484", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-administrativo-horario-flexible-remoto-1886769479", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H84" s="6" t="inlineStr"/>
@@ -4442,7 +4442,7 @@
     <row r="85" ht="22" customHeight="1">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>e4a3b83ad6ab6438</t>
+          <t>729fb015086632d9</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
@@ -4452,12 +4452,12 @@
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar administrativo(a) - licencia</t>
+          <t>Asistente de cuentas por pagar o tesoreria -remoto</t>
         </is>
       </c>
       <c r="D85" s="3" t="inlineStr">
         <is>
-          <t>FUCS</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E85" s="7" t="n">
@@ -4469,7 +4469,7 @@
         </is>
       </c>
       <c r="G85" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-administrativoa-licencia-1886759487", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/asistente-de-cuentas-por-pagar-o-tesoreria-remoto-1886744484", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H85" s="6" t="inlineStr"/>
@@ -4488,7 +4488,7 @@
     <row r="86" ht="22" customHeight="1">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2b1aa0caccddf7e4</t>
+          <t>e4a3b83ad6ab6438</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
@@ -4498,12 +4498,12 @@
       </c>
       <c r="C86" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar administrativo</t>
+          <t>Auxiliar administrativo(a) - licencia</t>
         </is>
       </c>
       <c r="D86" s="3" t="inlineStr">
         <is>
-          <t>Cruz Roja Colombiana Seccional Cundinamarca y Bogotá.</t>
+          <t>FUCS</t>
         </is>
       </c>
       <c r="E86" s="7" t="n">
@@ -4515,7 +4515,7 @@
         </is>
       </c>
       <c r="G86" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-administrativo-1886753336", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-administrativoa-licencia-1886759487", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H86" s="6" t="inlineStr"/>
@@ -4534,7 +4534,7 @@
     <row r="87" ht="22" customHeight="1">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>f864b0373b9419ab</t>
+          <t>2b1aa0caccddf7e4</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
@@ -4544,12 +4544,12 @@
       </c>
       <c r="C87" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar administrativo -ciencias basicas</t>
+          <t>Auxiliar administrativo</t>
         </is>
       </c>
       <c r="D87" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Cruz Roja Colombiana Seccional Cundinamarca y Bogotá.</t>
         </is>
       </c>
       <c r="E87" s="7" t="n">
@@ -4561,7 +4561,7 @@
         </is>
       </c>
       <c r="G87" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-administrativo-ciencias-basicas-1886759929", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-administrativo-1886753336", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H87" s="6" t="inlineStr"/>
@@ -4580,7 +4580,7 @@
     <row r="88" ht="22" customHeight="1">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>00a48d615f284d91</t>
+          <t>f864b0373b9419ab</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
@@ -4590,7 +4590,7 @@
       </c>
       <c r="C88" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar administrativo</t>
+          <t>Auxiliar administrativo -ciencias basicas</t>
         </is>
       </c>
       <c r="D88" s="3" t="inlineStr">
@@ -4607,7 +4607,7 @@
         </is>
       </c>
       <c r="G88" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-administrativo-bienestar-universitario-1886744996", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-administrativo-ciencias-basicas-1886759929", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H88" s="6" t="inlineStr"/>
@@ -4626,7 +4626,7 @@
     <row r="89" ht="22" customHeight="1">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>0544391db42d3941</t>
+          <t>00a48d615f284d91</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
@@ -4641,7 +4641,7 @@
       </c>
       <c r="D89" s="3" t="inlineStr">
         <is>
-          <t>FUCS</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E89" s="7" t="n">
@@ -4653,7 +4653,7 @@
         </is>
       </c>
       <c r="G89" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-administrativoa-1886769676", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-administrativo-bienestar-universitario-1886744996", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H89" s="6" t="inlineStr"/>
@@ -4672,7 +4672,7 @@
     <row r="90" ht="22" customHeight="1">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>e4338d6723631384</t>
+          <t>0544391db42d3941</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
@@ -4682,12 +4682,12 @@
       </c>
       <c r="C90" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar administrativo y de logística corporativa</t>
+          <t>Auxiliar administrativo</t>
         </is>
       </c>
       <c r="D90" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>FUCS</t>
         </is>
       </c>
       <c r="E90" s="7" t="n">
@@ -4699,7 +4699,7 @@
         </is>
       </c>
       <c r="G90" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-administrativo-y-de-logistica-corporativa-1886765843", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-administrativoa-1886769676", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H90" s="6" t="inlineStr"/>
@@ -4718,7 +4718,7 @@
     <row r="91" ht="22" customHeight="1">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>54d4c3f98f954a41</t>
+          <t>e4338d6723631384</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
@@ -4728,12 +4728,12 @@
       </c>
       <c r="C91" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar administrativo educación continua</t>
+          <t>Auxiliar administrativo y de logística corporativa</t>
         </is>
       </c>
       <c r="D91" s="3" t="inlineStr">
         <is>
-          <t>Fundación Santa Fe de Bogotá</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E91" s="7" t="n">
@@ -4745,7 +4745,7 @@
         </is>
       </c>
       <c r="G91" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-administrativo-educacion-continua-1886750214", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-administrativo-y-de-logistica-corporativa-1886765843", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H91" s="6" t="inlineStr"/>
@@ -4764,7 +4764,7 @@
     <row r="92" ht="22" customHeight="1">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>e824af898bf9a932</t>
+          <t>54d4c3f98f954a41</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
@@ -4774,12 +4774,12 @@
       </c>
       <c r="C92" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar administrativo y financiero</t>
+          <t>Auxiliar administrativo educación continua</t>
         </is>
       </c>
       <c r="D92" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Fundación Santa Fe de Bogotá</t>
         </is>
       </c>
       <c r="E92" s="7" t="n">
@@ -4791,7 +4791,7 @@
         </is>
       </c>
       <c r="G92" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-administrativo-y-financiero-1886753619", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-administrativo-educacion-continua-1886750214", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H92" s="6" t="inlineStr"/>
@@ -4810,7 +4810,7 @@
     <row r="93" ht="22" customHeight="1">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>54c86d8a0d796617</t>
+          <t>e824af898bf9a932</t>
         </is>
       </c>
       <c r="B93" s="2" t="inlineStr">
@@ -4820,12 +4820,12 @@
       </c>
       <c r="C93" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar administrativa</t>
+          <t>Auxiliar administrativo y financiero</t>
         </is>
       </c>
       <c r="D93" s="3" t="inlineStr">
         <is>
-          <t>ASISTALENTO SAS</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E93" s="7" t="n">
@@ -4837,7 +4837,7 @@
         </is>
       </c>
       <c r="G93" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-administrativa-1886767177", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-administrativo-y-financiero-1886753619", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H93" s="6" t="inlineStr"/>
@@ -4856,7 +4856,7 @@
     <row r="94" ht="22" customHeight="1">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>372b28276b98282f</t>
+          <t>54c86d8a0d796617</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
@@ -4866,12 +4866,12 @@
       </c>
       <c r="C94" s="3" t="inlineStr">
         <is>
-          <t>Secretaria administrativa</t>
+          <t>Auxiliar administrativa</t>
         </is>
       </c>
       <c r="D94" s="3" t="inlineStr">
         <is>
-          <t>FUNDACIÓN ANDES</t>
+          <t>ASISTALENTO SAS</t>
         </is>
       </c>
       <c r="E94" s="7" t="n">
@@ -4883,7 +4883,7 @@
         </is>
       </c>
       <c r="G94" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/secretaria-administrativa-1886756322", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-administrativa-1886767177", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H94" s="6" t="inlineStr"/>
@@ -4902,7 +4902,7 @@
     <row r="95" ht="22" customHeight="1">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>cee8b3db11750755</t>
+          <t>372b28276b98282f</t>
         </is>
       </c>
       <c r="B95" s="2" t="inlineStr">
@@ -4912,12 +4912,12 @@
       </c>
       <c r="C95" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar administrativo de obra</t>
+          <t>Secretaria administrativa</t>
         </is>
       </c>
       <c r="D95" s="3" t="inlineStr">
         <is>
-          <t>GRUPO AR S.A.</t>
+          <t>FUNDACIÓN ANDES</t>
         </is>
       </c>
       <c r="E95" s="7" t="n">
@@ -4929,7 +4929,7 @@
         </is>
       </c>
       <c r="G95" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-administrativo-de-obra-1886747241", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/secretaria-administrativa-1886756322", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H95" s="6" t="inlineStr"/>
@@ -4948,7 +4948,7 @@
     <row r="96" ht="22" customHeight="1">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>f86d411dd7ab31c0</t>
+          <t>cee8b3db11750755</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
@@ -4958,12 +4958,12 @@
       </c>
       <c r="C96" s="3" t="inlineStr">
         <is>
-          <t>Asistente administrativa supernumeraria</t>
+          <t>Auxiliar administrativo de obra</t>
         </is>
       </c>
       <c r="D96" s="3" t="inlineStr">
         <is>
-          <t>Grupo Good</t>
+          <t>GRUPO AR S.A.</t>
         </is>
       </c>
       <c r="E96" s="7" t="n">
@@ -4975,7 +4975,7 @@
         </is>
       </c>
       <c r="G96" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/asistente-administrativa-supernumeraria-1886762173", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-administrativo-de-obra-1886747241", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H96" s="6" t="inlineStr"/>
@@ -4994,7 +4994,7 @@
     <row r="97" ht="22" customHeight="1">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>02d246dd2c1d19fd</t>
+          <t>f86d411dd7ab31c0</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
@@ -5004,12 +5004,12 @@
       </c>
       <c r="C97" s="3" t="inlineStr">
         <is>
-          <t>Asistente ejecutiva</t>
+          <t>Asistente administrativa supernumeraria</t>
         </is>
       </c>
       <c r="D97" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Grupo Good</t>
         </is>
       </c>
       <c r="E97" s="7" t="n">
@@ -5021,7 +5021,7 @@
         </is>
       </c>
       <c r="G97" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/asistente-ejecutiva-1886745926", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/asistente-administrativa-supernumeraria-1886762173", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H97" s="6" t="inlineStr"/>
@@ -5040,7 +5040,7 @@
     <row r="98" ht="22" customHeight="1">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>b56bb36e9fc82e1e</t>
+          <t>02d246dd2c1d19fd</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
@@ -5050,12 +5050,12 @@
       </c>
       <c r="C98" s="3" t="inlineStr">
         <is>
-          <t>Asistente administrativo/a</t>
+          <t>Asistente ejecutiva</t>
         </is>
       </c>
       <c r="D98" s="3" t="inlineStr">
         <is>
-          <t>MEDICALL TALENTO HUMANO S.A.S.</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E98" s="7" t="n">
@@ -5067,7 +5067,7 @@
         </is>
       </c>
       <c r="G98" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/asistente-administrativo-a-1886747464", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/asistente-ejecutiva-1886745926", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H98" s="6" t="inlineStr"/>
@@ -5086,7 +5086,7 @@
     <row r="99" ht="22" customHeight="1">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>58fe156c45c49fc4</t>
+          <t>b56bb36e9fc82e1e</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
@@ -5096,12 +5096,12 @@
       </c>
       <c r="C99" s="3" t="inlineStr">
         <is>
-          <t>Asistente ejecutiva y personal de presidencia</t>
+          <t>Asistente administrativo/a</t>
         </is>
       </c>
       <c r="D99" s="3" t="inlineStr">
         <is>
-          <t>ADECCO COLOMBIA S A</t>
+          <t>MEDICALL TALENTO HUMANO S.A.S.</t>
         </is>
       </c>
       <c r="E99" s="7" t="n">
@@ -5113,7 +5113,7 @@
         </is>
       </c>
       <c r="G99" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/asistente-ejecutiva-y-personal-de-presidencia-1886765043", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/asistente-administrativo-a-1886747464", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H99" s="6" t="inlineStr"/>
@@ -5132,7 +5132,7 @@
     <row r="100" ht="22" customHeight="1">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>c68c842aec0507f5</t>
+          <t>58fe156c45c49fc4</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
@@ -5142,12 +5142,12 @@
       </c>
       <c r="C100" s="3" t="inlineStr">
         <is>
-          <t>Asistente administrativo y operativo</t>
+          <t>Asistente ejecutiva y personal de presidencia</t>
         </is>
       </c>
       <c r="D100" s="3" t="inlineStr">
         <is>
-          <t>ALIANZA</t>
+          <t>ADECCO COLOMBIA S A</t>
         </is>
       </c>
       <c r="E100" s="7" t="n">
@@ -5159,7 +5159,7 @@
         </is>
       </c>
       <c r="G100" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/asistente-administrativo-y-operativo-1886769341", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/asistente-ejecutiva-y-personal-de-presidencia-1886765043", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H100" s="6" t="inlineStr"/>
@@ -5178,7 +5178,7 @@
     <row r="101" ht="22" customHeight="1">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>e55c41f8f35d0d12</t>
+          <t>c68c842aec0507f5</t>
         </is>
       </c>
       <c r="B101" s="2" t="inlineStr">
@@ -5188,12 +5188,12 @@
       </c>
       <c r="C101" s="3" t="inlineStr">
         <is>
-          <t>Asistente administrativa y comercial pereira</t>
+          <t>Asistente administrativo y operativo</t>
         </is>
       </c>
       <c r="D101" s="3" t="inlineStr">
         <is>
-          <t>EDITORIAL LA REPÚBLICA S.A.S.</t>
+          <t>ALIANZA</t>
         </is>
       </c>
       <c r="E101" s="7" t="n">
@@ -5205,7 +5205,7 @@
         </is>
       </c>
       <c r="G101" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/asistente-administrativa-y-comercial-pereira-1886746894", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/asistente-administrativo-y-operativo-1886769341", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H101" s="6" t="inlineStr"/>
@@ -5224,7 +5224,7 @@
     <row r="102" ht="22" customHeight="1">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>0504d9833ad54912</t>
+          <t>e55c41f8f35d0d12</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
@@ -5234,12 +5234,12 @@
       </c>
       <c r="C102" s="3" t="inlineStr">
         <is>
-          <t>Asistente administrativo(a) at | bogotá</t>
+          <t>Asistente administrativa y comercial pereira</t>
         </is>
       </c>
       <c r="D102" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>EDITORIAL LA REPÚBLICA S.A.S.</t>
         </is>
       </c>
       <c r="E102" s="7" t="n">
@@ -5251,7 +5251,7 @@
         </is>
       </c>
       <c r="G102" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/asistente-administrativoa-at-bogota-1886765770", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/asistente-administrativa-y-comercial-pereira-1886746894", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H102" s="6" t="inlineStr"/>
@@ -5270,7 +5270,7 @@
     <row r="103" ht="22" customHeight="1">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>bacc38002882c624</t>
+          <t>0504d9833ad54912</t>
         </is>
       </c>
       <c r="B103" s="2" t="inlineStr">
@@ -5280,12 +5280,12 @@
       </c>
       <c r="C103" s="3" t="inlineStr">
         <is>
-          <t>Asistente administrativo</t>
+          <t>Asistente administrativo(a) at | bogotá</t>
         </is>
       </c>
       <c r="D103" s="3" t="inlineStr">
         <is>
-          <t>POSSE HERRERA Y RUIZ</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E103" s="7" t="n">
@@ -5297,7 +5297,7 @@
         </is>
       </c>
       <c r="G103" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/asistente-administrativo-1886757128", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/asistente-administrativoa-at-bogota-1886765770", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H103" s="6" t="inlineStr"/>
@@ -5316,7 +5316,7 @@
     <row r="104" ht="22" customHeight="1">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>115c420d4e627838</t>
+          <t>bacc38002882c624</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
@@ -5326,12 +5326,12 @@
       </c>
       <c r="C104" s="3" t="inlineStr">
         <is>
-          <t>Recepcionista y asistente administrativa</t>
+          <t>Asistente administrativo</t>
         </is>
       </c>
       <c r="D104" s="3" t="inlineStr">
         <is>
-          <t>Colliers International Colombia S.A</t>
+          <t>POSSE HERRERA Y RUIZ</t>
         </is>
       </c>
       <c r="E104" s="7" t="n">
@@ -5343,7 +5343,7 @@
         </is>
       </c>
       <c r="G104" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/recepcionista-y-asistente-administrativa-1886769882", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/asistente-administrativo-1886757128", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H104" s="6" t="inlineStr"/>
@@ -5362,7 +5362,7 @@
     <row r="105" ht="22" customHeight="1">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>0eafe890d09dc027</t>
+          <t>115c420d4e627838</t>
         </is>
       </c>
       <c r="B105" s="2" t="inlineStr">
@@ -5372,12 +5372,12 @@
       </c>
       <c r="C105" s="3" t="inlineStr">
         <is>
-          <t>Asistente administrativa y contable - chía | ref. 1626544466-1</t>
+          <t>Recepcionista y asistente administrativa</t>
         </is>
       </c>
       <c r="D105" s="3" t="inlineStr">
         <is>
-          <t>AGENCIA DE EMPLEO Y FOMENTO EMPRESARIAL COMPENSAR</t>
+          <t>Colliers International Colombia S.A</t>
         </is>
       </c>
       <c r="E105" s="7" t="n">
@@ -5389,7 +5389,7 @@
         </is>
       </c>
       <c r="G105" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/asistente-administrativa-y-contable-chia-ref-16265444661-1886766808", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/recepcionista-y-asistente-administrativa-1886769882", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H105" s="6" t="inlineStr"/>
@@ -5408,7 +5408,7 @@
     <row r="106" ht="22" customHeight="1">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>7fdb3ec2bb49ce90</t>
+          <t>0eafe890d09dc027</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
@@ -5418,12 +5418,12 @@
       </c>
       <c r="C106" s="3" t="inlineStr">
         <is>
-          <t>Asistente administrativa y contable</t>
+          <t>Asistente administrativa y contable - chía | ref. 1626544466-1</t>
         </is>
       </c>
       <c r="D106" s="3" t="inlineStr">
         <is>
-          <t>ASESORES FINANCIEROS Y TRIBUTARIOS GR SAS</t>
+          <t>AGENCIA DE EMPLEO Y FOMENTO EMPRESARIAL COMPENSAR</t>
         </is>
       </c>
       <c r="E106" s="7" t="n">
@@ -5435,7 +5435,7 @@
         </is>
       </c>
       <c r="G106" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/asistente-administrativa-y-contable-1886758421", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/asistente-administrativa-y-contable-chia-ref-16265444661-1886766808", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H106" s="6" t="inlineStr"/>
@@ -5454,7 +5454,7 @@
     <row r="107" ht="22" customHeight="1">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>08014f384f124ec4</t>
+          <t>7fdb3ec2bb49ce90</t>
         </is>
       </c>
       <c r="B107" s="2" t="inlineStr">
@@ -5464,12 +5464,12 @@
       </c>
       <c r="C107" s="3" t="inlineStr">
         <is>
-          <t>Asistente administrativo y contable - villeta</t>
+          <t>Asistente administrativa y contable</t>
         </is>
       </c>
       <c r="D107" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>ASESORES FINANCIEROS Y TRIBUTARIOS GR SAS</t>
         </is>
       </c>
       <c r="E107" s="7" t="n">
@@ -5481,7 +5481,7 @@
         </is>
       </c>
       <c r="G107" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/asistente-administrativo-y-contable-villeta-1886759076", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/asistente-administrativa-y-contable-1886758421", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H107" s="6" t="inlineStr"/>
@@ -5500,7 +5500,7 @@
     <row r="108" ht="22" customHeight="1">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>c62a542387886bca</t>
+          <t>08014f384f124ec4</t>
         </is>
       </c>
       <c r="B108" s="2" t="inlineStr">
@@ -5527,7 +5527,7 @@
         </is>
       </c>
       <c r="G108" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/asistente-administrativo-y-contable-villeta-1886758361", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/asistente-administrativo-y-contable-villeta-1886759076", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H108" s="6" t="inlineStr"/>
@@ -5546,7 +5546,7 @@
     <row r="109" ht="22" customHeight="1">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>fec983a79bc46288</t>
+          <t>c62a542387886bca</t>
         </is>
       </c>
       <c r="B109" s="2" t="inlineStr">
@@ -5556,12 +5556,12 @@
       </c>
       <c r="C109" s="3" t="inlineStr">
         <is>
-          <t>Asistente administrativo y contable</t>
+          <t>Asistente administrativo y contable - villeta</t>
         </is>
       </c>
       <c r="D109" s="3" t="inlineStr">
         <is>
-          <t>iLingo Integrated Solutions in Languages</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E109" s="7" t="n">
@@ -5573,7 +5573,7 @@
         </is>
       </c>
       <c r="G109" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/asistente-administrativo-y-contable-1886747606", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/asistente-administrativo-y-contable-villeta-1886758361", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H109" s="6" t="inlineStr"/>
@@ -5592,7 +5592,7 @@
     <row r="110" ht="22" customHeight="1">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>1871e0c68a13d38e</t>
+          <t>fec983a79bc46288</t>
         </is>
       </c>
       <c r="B110" s="2" t="inlineStr">
@@ -5602,12 +5602,12 @@
       </c>
       <c r="C110" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar contable - sap - bogota</t>
+          <t>Asistente administrativo y contable</t>
         </is>
       </c>
       <c r="D110" s="3" t="inlineStr">
         <is>
-          <t>ADECCO COLOMBIA S A</t>
+          <t>iLingo Integrated Solutions in Languages</t>
         </is>
       </c>
       <c r="E110" s="7" t="n">
@@ -5619,7 +5619,7 @@
         </is>
       </c>
       <c r="G110" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-contable-sap-bogota-1886767163", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/asistente-administrativo-y-contable-1886747606", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H110" s="6" t="inlineStr"/>
@@ -5638,7 +5638,7 @@
     <row r="111" ht="22" customHeight="1">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>6367348e3671a1aa</t>
+          <t>1871e0c68a13d38e</t>
         </is>
       </c>
       <c r="B111" s="2" t="inlineStr">
@@ -5648,12 +5648,12 @@
       </c>
       <c r="C111" s="3" t="inlineStr">
         <is>
-          <t>Asistente contable y administrativo con experiencia contable en sap, cartera y tesoreria</t>
+          <t>Auxiliar contable - sap - bogota</t>
         </is>
       </c>
       <c r="D111" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>ADECCO COLOMBIA S A</t>
         </is>
       </c>
       <c r="E111" s="7" t="n">
@@ -5665,7 +5665,7 @@
         </is>
       </c>
       <c r="G111" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/asistente-contable-y-administrativo-con-experiencia-contable-en-sap-cartera-y-tesoreria-1886760656", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-contable-sap-bogota-1886767163", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H111" s="6" t="inlineStr"/>
@@ -5684,7 +5684,7 @@
     <row r="112" ht="22" customHeight="1">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>fa85204cef58799f</t>
+          <t>6367348e3671a1aa</t>
         </is>
       </c>
       <c r="B112" s="2" t="inlineStr">
@@ -5694,7 +5694,7 @@
       </c>
       <c r="C112" s="3" t="inlineStr">
         <is>
-          <t>Asistente contable y administrativo con experiencia contable en sap - cartera y tesoreria</t>
+          <t>Asistente contable y administrativo con experiencia contable en sap, cartera y tesoreria</t>
         </is>
       </c>
       <c r="D112" s="3" t="inlineStr">
@@ -5711,7 +5711,7 @@
         </is>
       </c>
       <c r="G112" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/asistente-contable-y-administrativo-con-experiencia-contable-en-sap-cartera-y-tesoreria-1886766820", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/asistente-contable-y-administrativo-con-experiencia-contable-en-sap-cartera-y-tesoreria-1886760656", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H112" s="6" t="inlineStr"/>
@@ -5730,7 +5730,7 @@
     <row r="113" ht="22" customHeight="1">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>d8062d850cbf46a1</t>
+          <t>fa85204cef58799f</t>
         </is>
       </c>
       <c r="B113" s="2" t="inlineStr">
@@ -5740,12 +5740,12 @@
       </c>
       <c r="C113" s="3" t="inlineStr">
         <is>
-          <t>Digitador - 353703-113642</t>
+          <t>Asistente contable y administrativo con experiencia contable en sap - cartera y tesoreria</t>
         </is>
       </c>
       <c r="D113" s="3" t="inlineStr">
         <is>
-          <t>AGENCIA DE EMPLEO Y FOMENTO EMPRESARIAL COMPENSAR</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E113" s="7" t="n">
@@ -5757,7 +5757,7 @@
         </is>
       </c>
       <c r="G113" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/digitador-353703113642-1886769566", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/asistente-contable-y-administrativo-con-experiencia-contable-en-sap-cartera-y-tesoreria-1886766820", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H113" s="6" t="inlineStr"/>
@@ -5776,7 +5776,7 @@
     <row r="114" ht="22" customHeight="1">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>2f520ba083e2847f</t>
+          <t>d8062d850cbf46a1</t>
         </is>
       </c>
       <c r="B114" s="2" t="inlineStr">
@@ -5786,12 +5786,12 @@
       </c>
       <c r="C114" s="3" t="inlineStr">
         <is>
-          <t>Digitador en planta de producción</t>
+          <t>Digitador - 353703-113642</t>
         </is>
       </c>
       <c r="D114" s="3" t="inlineStr">
         <is>
-          <t>Prysmian Group - Procables</t>
+          <t>AGENCIA DE EMPLEO Y FOMENTO EMPRESARIAL COMPENSAR</t>
         </is>
       </c>
       <c r="E114" s="7" t="n">
@@ -5803,7 +5803,7 @@
         </is>
       </c>
       <c r="G114" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/digitador-en-planta-de-produccion-1886722751", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/digitador-353703113642-1886769566", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H114" s="6" t="inlineStr"/>
@@ -5822,7 +5822,7 @@
     <row r="115" ht="22" customHeight="1">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>475f3966c5302ff0</t>
+          <t>2f520ba083e2847f</t>
         </is>
       </c>
       <c r="B115" s="2" t="inlineStr">
@@ -5832,12 +5832,12 @@
       </c>
       <c r="C115" s="3" t="inlineStr">
         <is>
-          <t>Analista de aduana - digitador opencomex</t>
+          <t>Digitador en planta de producción</t>
         </is>
       </c>
       <c r="D115" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Prysmian Group - Procables</t>
         </is>
       </c>
       <c r="E115" s="7" t="n">
@@ -5849,7 +5849,7 @@
         </is>
       </c>
       <c r="G115" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-aduana-digitador-opencomex-1886762323", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/digitador-en-planta-de-produccion-1886722751", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H115" s="6" t="inlineStr"/>
@@ -5868,7 +5868,7 @@
     <row r="116" ht="22" customHeight="1">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>107d0765b8dfce86</t>
+          <t>475f3966c5302ff0</t>
         </is>
       </c>
       <c r="B116" s="2" t="inlineStr">
@@ -5878,7 +5878,7 @@
       </c>
       <c r="C116" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar digitador(a) de contabilidad</t>
+          <t>Analista de aduana - digitador opencomex</t>
         </is>
       </c>
       <c r="D116" s="3" t="inlineStr">
@@ -5895,7 +5895,7 @@
         </is>
       </c>
       <c r="G116" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-digitadora-de-contabilidad-1886770758", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-aduana-digitador-opencomex-1886762323", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H116" s="6" t="inlineStr"/>
@@ -5914,7 +5914,7 @@
     <row r="117" ht="22" customHeight="1">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>b1591783dbbcb1f9</t>
+          <t>107d0765b8dfce86</t>
         </is>
       </c>
       <c r="B117" s="2" t="inlineStr">
@@ -5924,7 +5924,7 @@
       </c>
       <c r="C117" s="3" t="inlineStr">
         <is>
-          <t>Analista de aduana - digitador opencomex</t>
+          <t>Auxiliar digitador(a) de contabilidad</t>
         </is>
       </c>
       <c r="D117" s="3" t="inlineStr">
@@ -5941,7 +5941,7 @@
         </is>
       </c>
       <c r="G117" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-aduana-digitador-opencomex-1886763468", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-digitadora-de-contabilidad-1886770758", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H117" s="6" t="inlineStr"/>
@@ -5960,7 +5960,7 @@
     <row r="118" ht="22" customHeight="1">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>cfe8b8276b28373b</t>
+          <t>b1591783dbbcb1f9</t>
         </is>
       </c>
       <c r="B118" s="2" t="inlineStr">
@@ -5970,7 +5970,7 @@
       </c>
       <c r="C118" s="3" t="inlineStr">
         <is>
-          <t>Analista de aduana - digitador opencomex - santa marta</t>
+          <t>Analista de aduana - digitador opencomex</t>
         </is>
       </c>
       <c r="D118" s="3" t="inlineStr">
@@ -5987,7 +5987,7 @@
         </is>
       </c>
       <c r="G118" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-aduana-digitador-opencomex-santa-marta-1886762869", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-aduana-digitador-opencomex-1886763468", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H118" s="6" t="inlineStr"/>
@@ -6006,7 +6006,7 @@
     <row r="119" ht="22" customHeight="1">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>01c7ac97b62a3626</t>
+          <t>cfe8b8276b28373b</t>
         </is>
       </c>
       <c r="B119" s="2" t="inlineStr">
@@ -6016,7 +6016,7 @@
       </c>
       <c r="C119" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar digitador(a) de contabilidad</t>
+          <t>Analista de aduana - digitador opencomex - santa marta</t>
         </is>
       </c>
       <c r="D119" s="3" t="inlineStr">
@@ -6033,7 +6033,7 @@
         </is>
       </c>
       <c r="G119" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-digitadora-de-contabilidad-1886761791", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-aduana-digitador-opencomex-santa-marta-1886762869", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H119" s="6" t="inlineStr"/>
@@ -6052,7 +6052,7 @@
     <row r="120" ht="22" customHeight="1">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>2fc59d447ad455e1</t>
+          <t>01c7ac97b62a3626</t>
         </is>
       </c>
       <c r="B120" s="2" t="inlineStr">
@@ -6062,12 +6062,12 @@
       </c>
       <c r="C120" s="3" t="inlineStr">
         <is>
-          <t>Digitador comercial interno</t>
+          <t>Auxiliar digitador(a) de contabilidad</t>
         </is>
       </c>
       <c r="D120" s="3" t="inlineStr">
         <is>
-          <t>TEMPORIZAR SERVICIOS TEMPORALES SAS</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E120" s="7" t="n">
@@ -6079,7 +6079,7 @@
         </is>
       </c>
       <c r="G120" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/digitador-comercial-interno-1886746080", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-digitadora-de-contabilidad-1886761791", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H120" s="6" t="inlineStr"/>
@@ -6098,7 +6098,7 @@
     <row r="121" ht="22" customHeight="1">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>e58059d4e095bd7a</t>
+          <t>2fc59d447ad455e1</t>
         </is>
       </c>
       <c r="B121" s="2" t="inlineStr">
@@ -6108,12 +6108,12 @@
       </c>
       <c r="C121" s="3" t="inlineStr">
         <is>
-          <t>Apoyo facturación - palmira</t>
+          <t>Digitador comercial interno</t>
         </is>
       </c>
       <c r="D121" s="3" t="inlineStr">
         <is>
-          <t>ALQUERIA</t>
+          <t>TEMPORIZAR SERVICIOS TEMPORALES SAS</t>
         </is>
       </c>
       <c r="E121" s="7" t="n">
@@ -6125,13 +6125,13 @@
         </is>
       </c>
       <c r="G121" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/apoyo-facturacion-palmira-1886758686", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/digitador-comercial-interno-1886746080", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H121" s="6" t="inlineStr"/>
       <c r="I121" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Alta coincidencia técnica en Herramientas Ofimáticas, Excel y Soporte Contable / Facturación. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Auxiliar Administrativo / Asistente Virtual). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J121" s="2" t="inlineStr">
@@ -6144,7 +6144,7 @@
     <row r="122" ht="22" customHeight="1">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>62e7c31c63a388da</t>
+          <t>e58059d4e095bd7a</t>
         </is>
       </c>
       <c r="B122" s="2" t="inlineStr">
@@ -6154,12 +6154,12 @@
       </c>
       <c r="C122" s="3" t="inlineStr">
         <is>
-          <t>Recepcion y facturacion de laboratorio clínico</t>
+          <t>Apoyo facturación - palmira</t>
         </is>
       </c>
       <c r="D122" s="3" t="inlineStr">
         <is>
-          <t>Fundación Santa Fe de Bogotá</t>
+          <t>ALQUERIA</t>
         </is>
       </c>
       <c r="E122" s="7" t="n">
@@ -6171,7 +6171,7 @@
         </is>
       </c>
       <c r="G122" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/recepcion-y-facturacion-de-laboratorio-clinico-1886761193", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/apoyo-facturacion-palmira-1886758686", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H122" s="6" t="inlineStr"/>
@@ -6190,7 +6190,7 @@
     <row r="123" ht="22" customHeight="1">
       <c r="A123" s="2" t="inlineStr">
         <is>
-          <t>6eafefaa9d4e76e6</t>
+          <t>62e7c31c63a388da</t>
         </is>
       </c>
       <c r="B123" s="2" t="inlineStr">
@@ -6200,7 +6200,7 @@
       </c>
       <c r="C123" s="3" t="inlineStr">
         <is>
-          <t>Recepcionista facturación en laboratorio clínico</t>
+          <t>Recepcion y facturacion de laboratorio clínico</t>
         </is>
       </c>
       <c r="D123" s="3" t="inlineStr">
@@ -6217,7 +6217,7 @@
         </is>
       </c>
       <c r="G123" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/recepcionista-facturacion-en-laboratorio-clinico-1886753959", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/recepcion-y-facturacion-de-laboratorio-clinico-1886761193", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H123" s="6" t="inlineStr"/>
@@ -6236,7 +6236,7 @@
     <row r="124" ht="22" customHeight="1">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>1ac2af8aa1b80d19</t>
+          <t>6eafefaa9d4e76e6</t>
         </is>
       </c>
       <c r="B124" s="2" t="inlineStr">
@@ -6263,7 +6263,7 @@
         </is>
       </c>
       <c r="G124" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/recepcionista-facturacion-en-laboratorio-clinico-1886746927", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/recepcionista-facturacion-en-laboratorio-clinico-1886753959", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H124" s="6" t="inlineStr"/>
@@ -6282,7 +6282,7 @@
     <row r="125" ht="22" customHeight="1">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t>5fb21eaeba4e417d</t>
+          <t>1ac2af8aa1b80d19</t>
         </is>
       </c>
       <c r="B125" s="2" t="inlineStr">
@@ -6292,12 +6292,12 @@
       </c>
       <c r="C125" s="3" t="inlineStr">
         <is>
-          <t>Gestor de Facturación e Ingresos // Remoto</t>
+          <t>Recepcionista facturación en laboratorio clínico</t>
         </is>
       </c>
       <c r="D125" s="3" t="inlineStr">
         <is>
-          <t>Siigo</t>
+          <t>Fundación Santa Fe de Bogotá</t>
         </is>
       </c>
       <c r="E125" s="7" t="n">
@@ -6309,7 +6309,7 @@
         </is>
       </c>
       <c r="G125" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/gestor-de-facturaci%C3%B3n-e-ingresos-remoto-pcd-at-siigo-4463333674", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/recepcionista-facturacion-en-laboratorio-clinico-1886746927", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H125" s="6" t="inlineStr"/>
@@ -6328,7 +6328,7 @@
     <row r="126" ht="22" customHeight="1">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>acc279cbcc202e8c</t>
+          <t>5fb21eaeba4e417d</t>
         </is>
       </c>
       <c r="B126" s="2" t="inlineStr">
@@ -6338,12 +6338,12 @@
       </c>
       <c r="C126" s="3" t="inlineStr">
         <is>
-          <t>Data Entry Clerk</t>
+          <t>Gestor de Facturación e Ingresos // Remoto</t>
         </is>
       </c>
       <c r="D126" s="3" t="inlineStr">
         <is>
-          <t>Hired</t>
+          <t>Siigo</t>
         </is>
       </c>
       <c r="E126" s="7" t="n">
@@ -6355,13 +6355,13 @@
         </is>
       </c>
       <c r="G126" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/data-entry-clerk-remote-at-hired-4466319108", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/gestor-de-facturaci%C3%B3n-e-ingresos-remoto-pcd-at-siigo-4463333674", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H126" s="6" t="inlineStr"/>
       <c r="I126" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Auxiliar Administrativo / Asistente Virtual). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Alta coincidencia técnica en Herramientas Ofimáticas, Excel y Soporte Contable / Facturación. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J126" s="2" t="inlineStr">
@@ -6374,7 +6374,7 @@
     <row r="127" ht="22" customHeight="1">
       <c r="A127" s="2" t="inlineStr">
         <is>
-          <t>c9df64f69713d9c3</t>
+          <t>acc279cbcc202e8c</t>
         </is>
       </c>
       <c r="B127" s="2" t="inlineStr">
@@ -6384,12 +6384,12 @@
       </c>
       <c r="C127" s="3" t="inlineStr">
         <is>
-          <t>Client Intake and Data Entry Specialist</t>
+          <t>Data Entry Clerk</t>
         </is>
       </c>
       <c r="D127" s="3" t="inlineStr">
         <is>
-          <t>Job Duck</t>
+          <t>Hired</t>
         </is>
       </c>
       <c r="E127" s="7" t="n">
@@ -6401,7 +6401,7 @@
         </is>
       </c>
       <c r="G127" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/client-intake-and-data-entry-specialist-at-job-duck-4469179215", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/data-entry-clerk-remote-at-hired-4466319108", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H127" s="6" t="inlineStr"/>
@@ -6420,7 +6420,7 @@
     <row r="128" ht="22" customHeight="1">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>bfd4f2e4c8eb51d6</t>
+          <t>c9df64f69713d9c3</t>
         </is>
       </c>
       <c r="B128" s="2" t="inlineStr">
@@ -6430,12 +6430,12 @@
       </c>
       <c r="C128" s="3" t="inlineStr">
         <is>
-          <t>Data Entry Specialist - Remote Work | REF#169097</t>
+          <t>Client Intake and Data Entry Specialist</t>
         </is>
       </c>
       <c r="D128" s="3" t="inlineStr">
         <is>
-          <t>BairesDev</t>
+          <t>Job Duck</t>
         </is>
       </c>
       <c r="E128" s="7" t="n">
@@ -6447,7 +6447,7 @@
         </is>
       </c>
       <c r="G128" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/data-entry-specialist-remote-work-ref%23169097-at-bairesdev-4140196697", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/client-intake-and-data-entry-specialist-at-job-duck-4469179215", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H128" s="6" t="inlineStr"/>
@@ -6466,7 +6466,7 @@
     <row r="129" ht="22" customHeight="1">
       <c r="A129" s="2" t="inlineStr">
         <is>
-          <t>f71b85e853980a5b</t>
+          <t>bfd4f2e4c8eb51d6</t>
         </is>
       </c>
       <c r="B129" s="2" t="inlineStr">
@@ -6476,12 +6476,12 @@
       </c>
       <c r="C129" s="3" t="inlineStr">
         <is>
-          <t>Data Entry Specialist</t>
+          <t>Data Entry Specialist - Remote Work | REF#169097</t>
         </is>
       </c>
       <c r="D129" s="3" t="inlineStr">
         <is>
-          <t>Booth</t>
+          <t>BairesDev</t>
         </is>
       </c>
       <c r="E129" s="7" t="n">
@@ -6493,7 +6493,7 @@
         </is>
       </c>
       <c r="G129" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/data-entry-specialist-at-booth-4468950013", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/data-entry-specialist-remote-work-ref%23169097-at-bairesdev-4140196697", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H129" s="6" t="inlineStr"/>
@@ -6512,7 +6512,7 @@
     <row r="130" ht="22" customHeight="1">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>b124540f32e77f79</t>
+          <t>f71b85e853980a5b</t>
         </is>
       </c>
       <c r="B130" s="2" t="inlineStr">
@@ -6522,12 +6522,12 @@
       </c>
       <c r="C130" s="3" t="inlineStr">
         <is>
-          <t>Digitador</t>
+          <t>Data Entry Specialist</t>
         </is>
       </c>
       <c r="D130" s="3" t="inlineStr">
         <is>
-          <t>Iron Mountain</t>
+          <t>Booth</t>
         </is>
       </c>
       <c r="E130" s="7" t="n">
@@ -6539,7 +6539,7 @@
         </is>
       </c>
       <c r="G130" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/digitador-at-iron-mountain-4468884742", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/data-entry-specialist-at-booth-4468950013", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H130" s="6" t="inlineStr"/>
@@ -6558,7 +6558,7 @@
     <row r="131" ht="22" customHeight="1">
       <c r="A131" s="2" t="inlineStr">
         <is>
-          <t>648f264595161cd7</t>
+          <t>b124540f32e77f79</t>
         </is>
       </c>
       <c r="B131" s="2" t="inlineStr">
@@ -6568,12 +6568,12 @@
       </c>
       <c r="C131" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar Administrativa de Vicepresidencia Bilingüe</t>
+          <t>Digitador</t>
         </is>
       </c>
       <c r="D131" s="3" t="inlineStr">
         <is>
-          <t>Adecco</t>
+          <t>Iron Mountain</t>
         </is>
       </c>
       <c r="E131" s="7" t="n">
@@ -6585,7 +6585,7 @@
         </is>
       </c>
       <c r="G131" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/auxiliar-administrativa-de-vicepresidencia-biling%C3%BCe-at-adecco-4469224990", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/digitador-at-iron-mountain-4468884742", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H131" s="6" t="inlineStr"/>
@@ -6604,7 +6604,7 @@
     <row r="132" ht="22" customHeight="1">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>eb90ed56020b1176</t>
+          <t>648f264595161cd7</t>
         </is>
       </c>
       <c r="B132" s="2" t="inlineStr">
@@ -6614,12 +6614,12 @@
       </c>
       <c r="C132" s="3" t="inlineStr">
         <is>
-          <t>Inside Sales Contractor</t>
+          <t>Auxiliar Administrativa de Vicepresidencia Bilingüe</t>
         </is>
       </c>
       <c r="D132" s="3" t="inlineStr">
         <is>
-          <t>Credit Wellness, LLC</t>
+          <t>Adecco</t>
         </is>
       </c>
       <c r="E132" s="7" t="n">
@@ -6631,17 +6631,13 @@
         </is>
       </c>
       <c r="G132" s="5">
-        <f>HYPERLINK("https://remotive.com/remote-jobs/sales/inside-sales-contractor-2086540", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H132" s="6" t="inlineStr">
-        <is>
-          <t>OTE $25k - $35k</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/auxiliar-administrativa-de-vicepresidencia-biling%C3%BCe-at-adecco-4469224990", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H132" s="6" t="inlineStr"/>
       <c r="I132" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Alta coincidencia técnica en Herramientas Ofimáticas, Excel y Soporte Contable / Facturación. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Auxiliar Administrativo / Asistente Virtual). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J132" s="2" t="inlineStr">
@@ -6654,22 +6650,22 @@
     <row r="133" ht="22" customHeight="1">
       <c r="A133" s="2" t="inlineStr">
         <is>
-          <t>ebabcd51596d0d3b</t>
+          <t>eb90ed56020b1176</t>
         </is>
       </c>
       <c r="B133" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 15:56</t>
+          <t>2026-09-24 16:07</t>
         </is>
       </c>
       <c r="C133" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar contable y administrativo</t>
+          <t>Inside Sales Contractor</t>
         </is>
       </c>
       <c r="D133" s="3" t="inlineStr">
         <is>
-          <t>ACTIVE ACCOUNTING GROUP</t>
+          <t>Credit Wellness, LLC</t>
         </is>
       </c>
       <c r="E133" s="7" t="n">
@@ -6681,17 +6677,17 @@
         </is>
       </c>
       <c r="G133" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-contable-y-administrativo-con-experiencia-en-el-santuario-C71D6812AE6D474061373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://remotive.com/remote-jobs/sales/inside-sales-contractor-2086540", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H133" s="6" t="inlineStr">
         <is>
-          <t>$ 1.750.905,00 (Mensual)</t>
+          <t>OTE $25k - $35k</t>
         </is>
       </c>
       <c r="I133" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Auxiliar Administrativo / Asistente Virtual). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Alta coincidencia técnica en Herramientas Ofimáticas, Excel y Soporte Contable / Facturación. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J133" s="2" t="inlineStr">
@@ -6704,7 +6700,7 @@
     <row r="134" ht="22" customHeight="1">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>e12bdf1aa280de03</t>
+          <t>ebabcd51596d0d3b</t>
         </is>
       </c>
       <c r="B134" s="2" t="inlineStr">
@@ -6714,12 +6710,12 @@
       </c>
       <c r="C134" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar administrativo</t>
+          <t>Auxiliar contable y administrativo</t>
         </is>
       </c>
       <c r="D134" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>ACTIVE ACCOUNTING GROUP</t>
         </is>
       </c>
       <c r="E134" s="7" t="n">
@@ -6731,10 +6727,14 @@
         </is>
       </c>
       <c r="G134" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-administrativoa-1886768459", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H134" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-contable-y-administrativo-con-experiencia-en-el-santuario-C71D6812AE6D474061373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H134" s="6" t="inlineStr">
+        <is>
+          <t>$ 1.750.905,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I134" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Auxiliar Administrativo / Asistente Virtual). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -6750,7 +6750,7 @@
     <row r="135" ht="22" customHeight="1">
       <c r="A135" s="2" t="inlineStr">
         <is>
-          <t>b1fccbf6d15bddc2</t>
+          <t>e12bdf1aa280de03</t>
         </is>
       </c>
       <c r="B135" s="2" t="inlineStr">
@@ -6760,12 +6760,12 @@
       </c>
       <c r="C135" s="3" t="inlineStr">
         <is>
-          <t>Asistente administrativa</t>
+          <t>Auxiliar administrativo</t>
         </is>
       </c>
       <c r="D135" s="3" t="inlineStr">
         <is>
-          <t>Dra Lina Bedoya Odontologia Estetica</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E135" s="7" t="n">
@@ -6777,7 +6777,7 @@
         </is>
       </c>
       <c r="G135" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/asistente-administrativa-1886766293", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-administrativoa-1886768459", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H135" s="6" t="inlineStr"/>
@@ -6796,7 +6796,7 @@
     <row r="136" ht="22" customHeight="1">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>db6a52513ae159ab</t>
+          <t>b1fccbf6d15bddc2</t>
         </is>
       </c>
       <c r="B136" s="2" t="inlineStr">
@@ -6806,12 +6806,12 @@
       </c>
       <c r="C136" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar contable - sap - bogota</t>
+          <t>Asistente administrativa</t>
         </is>
       </c>
       <c r="D136" s="3" t="inlineStr">
         <is>
-          <t>ADECCO COLOMBIA S A</t>
+          <t>Dra Lina Bedoya Odontologia Estetica</t>
         </is>
       </c>
       <c r="E136" s="7" t="n">
@@ -6823,7 +6823,7 @@
         </is>
       </c>
       <c r="G136" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-contable-sap-bogota-1886767591", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/asistente-administrativa-1886766293", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H136" s="6" t="inlineStr"/>
@@ -6842,7 +6842,7 @@
     <row r="137" ht="22" customHeight="1">
       <c r="A137" s="2" t="inlineStr">
         <is>
-          <t>ae9358eb43bb2f5b</t>
+          <t>db6a52513ae159ab</t>
         </is>
       </c>
       <c r="B137" s="2" t="inlineStr">
@@ -6869,7 +6869,7 @@
         </is>
       </c>
       <c r="G137" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-contable-sap-bogota-1886767165", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-contable-sap-bogota-1886767591", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H137" s="6" t="inlineStr"/>
@@ -6888,7 +6888,7 @@
     <row r="138" ht="22" customHeight="1">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t>daa8b5315dfb38c2</t>
+          <t>ae9358eb43bb2f5b</t>
         </is>
       </c>
       <c r="B138" s="2" t="inlineStr">
@@ -6915,7 +6915,7 @@
         </is>
       </c>
       <c r="G138" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-contable-sap-bogota-1886767164", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-contable-sap-bogota-1886767165", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H138" s="6" t="inlineStr"/>
@@ -6934,7 +6934,7 @@
     <row r="139" ht="22" customHeight="1">
       <c r="A139" s="2" t="inlineStr">
         <is>
-          <t>2d35aa26ef7d8409</t>
+          <t>daa8b5315dfb38c2</t>
         </is>
       </c>
       <c r="B139" s="2" t="inlineStr">
@@ -6944,12 +6944,12 @@
       </c>
       <c r="C139" s="3" t="inlineStr">
         <is>
-          <t>Almacenista digitador</t>
+          <t>Auxiliar contable - sap - bogota</t>
         </is>
       </c>
       <c r="D139" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>ADECCO COLOMBIA S A</t>
         </is>
       </c>
       <c r="E139" s="7" t="n">
@@ -6961,7 +6961,7 @@
         </is>
       </c>
       <c r="G139" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/almacenista-digitador-1886754273", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-contable-sap-bogota-1886767164", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H139" s="6" t="inlineStr"/>
@@ -6980,7 +6980,7 @@
     <row r="140" ht="22" customHeight="1">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t>a36cc8c2293d75bb</t>
+          <t>2d35aa26ef7d8409</t>
         </is>
       </c>
       <c r="B140" s="2" t="inlineStr">
@@ -6990,12 +6990,12 @@
       </c>
       <c r="C140" s="3" t="inlineStr">
         <is>
-          <t>Aux de facturacion - personas con discapacidad - bogota</t>
+          <t>Almacenista digitador</t>
         </is>
       </c>
       <c r="D140" s="3" t="inlineStr">
         <is>
-          <t>Quirón Prevención Colombia S.A.S</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E140" s="7" t="n">
@@ -7007,13 +7007,13 @@
         </is>
       </c>
       <c r="G140" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/aux-de-facturacion-personas-con-discapacidad-bogota-1886768842", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/almacenista-digitador-1886754273", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H140" s="6" t="inlineStr"/>
       <c r="I140" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Alta coincidencia técnica en Herramientas Ofimáticas, Excel y Soporte Contable / Facturación. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Auxiliar Administrativo / Asistente Virtual). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J140" s="2" t="inlineStr">
@@ -7026,7 +7026,7 @@
     <row r="141" ht="22" customHeight="1">
       <c r="A141" s="2" t="inlineStr">
         <is>
-          <t>e482852a389226cd</t>
+          <t>a36cc8c2293d75bb</t>
         </is>
       </c>
       <c r="B141" s="2" t="inlineStr">
@@ -7036,12 +7036,12 @@
       </c>
       <c r="C141" s="3" t="inlineStr">
         <is>
-          <t>Ejecutivo de cuenta / facturación electrónica</t>
+          <t>Aux de facturacion - personas con discapacidad - bogota</t>
         </is>
       </c>
       <c r="D141" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Quirón Prevención Colombia S.A.S</t>
         </is>
       </c>
       <c r="E141" s="7" t="n">
@@ -7053,7 +7053,7 @@
         </is>
       </c>
       <c r="G141" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/ejecutivo-de-cuenta-facturacion-electronica-1886754585", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/aux-de-facturacion-personas-con-discapacidad-bogota-1886768842", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H141" s="6" t="inlineStr"/>
@@ -7072,7 +7072,7 @@
     <row r="142" ht="22" customHeight="1">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t>0dfab7dcd9959d45</t>
+          <t>e482852a389226cd</t>
         </is>
       </c>
       <c r="B142" s="2" t="inlineStr">
@@ -7082,12 +7082,12 @@
       </c>
       <c r="C142" s="3" t="inlineStr">
         <is>
-          <t>Recepcion y facturacion de laboratorio clínico</t>
+          <t>Ejecutivo de cuenta / facturación electrónica</t>
         </is>
       </c>
       <c r="D142" s="3" t="inlineStr">
         <is>
-          <t>Fundación Santa Fe de Bogotá</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E142" s="7" t="n">
@@ -7099,7 +7099,7 @@
         </is>
       </c>
       <c r="G142" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/recepcion-y-facturacion-de-laboratorio-clinico-1886771931", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/ejecutivo-de-cuenta-facturacion-electronica-1886754585", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H142" s="6" t="inlineStr"/>
@@ -7118,22 +7118,22 @@
     <row r="143" ht="22" customHeight="1">
       <c r="A143" s="2" t="inlineStr">
         <is>
-          <t>f89540ec077787b1</t>
+          <t>0dfab7dcd9959d45</t>
         </is>
       </c>
       <c r="B143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26 15:05</t>
+          <t>2026-09-25 15:56</t>
         </is>
       </c>
       <c r="C143" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar administrativo</t>
+          <t>Recepcion y facturacion de laboratorio clínico</t>
         </is>
       </c>
       <c r="D143" s="3" t="inlineStr">
         <is>
-          <t>FUCS</t>
+          <t>Fundación Santa Fe de Bogotá</t>
         </is>
       </c>
       <c r="E143" s="7" t="n">
@@ -7145,13 +7145,13 @@
         </is>
       </c>
       <c r="G143" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-administrativoa-1886772558", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/recepcion-y-facturacion-de-laboratorio-clinico-1886771931", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H143" s="6" t="inlineStr"/>
       <c r="I143" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Auxiliar Administrativo / Asistente Virtual). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Alta coincidencia técnica en Herramientas Ofimáticas, Excel y Soporte Contable / Facturación. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J143" s="2" t="inlineStr">
@@ -7164,7 +7164,7 @@
     <row r="144" ht="22" customHeight="1">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>abffa88133eaa978</t>
+          <t>f89540ec077787b1</t>
         </is>
       </c>
       <c r="B144" s="2" t="inlineStr">
@@ -7174,12 +7174,12 @@
       </c>
       <c r="C144" s="3" t="inlineStr">
         <is>
-          <t>Almacenista digitador</t>
+          <t>Auxiliar administrativo</t>
         </is>
       </c>
       <c r="D144" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>FUCS</t>
         </is>
       </c>
       <c r="E144" s="7" t="n">
@@ -7191,7 +7191,7 @@
         </is>
       </c>
       <c r="G144" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/almacenista-digitador-1886749637", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-administrativoa-1886772558", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H144" s="6" t="inlineStr"/>
@@ -7210,7 +7210,7 @@
     <row r="145" ht="22" customHeight="1">
       <c r="A145" s="2" t="inlineStr">
         <is>
-          <t>e4ad43c355211b6e</t>
+          <t>abffa88133eaa978</t>
         </is>
       </c>
       <c r="B145" s="2" t="inlineStr">
@@ -7220,12 +7220,12 @@
       </c>
       <c r="C145" s="3" t="inlineStr">
         <is>
-          <t>Aux de facturacion - personas con discapacidad - bogota</t>
+          <t>Almacenista digitador</t>
         </is>
       </c>
       <c r="D145" s="3" t="inlineStr">
         <is>
-          <t>Quirón Prevención Colombia S.A.S</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E145" s="7" t="n">
@@ -7237,13 +7237,13 @@
         </is>
       </c>
       <c r="G145" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/aux-de-facturacion-personas-con-discapacidad-bogota-1886772337", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/almacenista-digitador-1886749637", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H145" s="6" t="inlineStr"/>
       <c r="I145" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Alta coincidencia técnica en Herramientas Ofimáticas, Excel y Soporte Contable / Facturación. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Auxiliar Administrativo / Asistente Virtual). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J145" s="2" t="inlineStr">
@@ -7256,7 +7256,7 @@
     <row r="146" ht="22" customHeight="1">
       <c r="A146" s="2" t="inlineStr">
         <is>
-          <t>ebfb9e3d2b3f916c</t>
+          <t>e4ad43c355211b6e</t>
         </is>
       </c>
       <c r="B146" s="2" t="inlineStr">
@@ -7266,12 +7266,12 @@
       </c>
       <c r="C146" s="3" t="inlineStr">
         <is>
-          <t>Recepcion y facturacion de laboratorio clínico</t>
+          <t>Aux de facturacion - personas con discapacidad - bogota</t>
         </is>
       </c>
       <c r="D146" s="3" t="inlineStr">
         <is>
-          <t>Fundación Santa Fe de Bogotá</t>
+          <t>Quirón Prevención Colombia S.A.S</t>
         </is>
       </c>
       <c r="E146" s="7" t="n">
@@ -7283,7 +7283,7 @@
         </is>
       </c>
       <c r="G146" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/recepcion-y-facturacion-de-laboratorio-clinico-1886767371", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/aux-de-facturacion-personas-con-discapacidad-bogota-1886772337", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H146" s="6" t="inlineStr"/>
@@ -7302,7 +7302,7 @@
     <row r="147" ht="22" customHeight="1">
       <c r="A147" s="2" t="inlineStr">
         <is>
-          <t>8478e893d783ed5e</t>
+          <t>ebfb9e3d2b3f916c</t>
         </is>
       </c>
       <c r="B147" s="2" t="inlineStr">
@@ -7312,7 +7312,7 @@
       </c>
       <c r="C147" s="3" t="inlineStr">
         <is>
-          <t>Recepcion y facturacion de laboratorio clinico</t>
+          <t>Recepcion y facturacion de laboratorio clínico</t>
         </is>
       </c>
       <c r="D147" s="3" t="inlineStr">
@@ -7329,7 +7329,7 @@
         </is>
       </c>
       <c r="G147" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/recepcion-y-facturacion-de-laboratorio-clinico-1886760903", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/recepcion-y-facturacion-de-laboratorio-clinico-1886767371", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H147" s="6" t="inlineStr"/>
@@ -7348,7 +7348,7 @@
     <row r="148" ht="22" customHeight="1">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>d45621f8599206ec</t>
+          <t>8478e893d783ed5e</t>
         </is>
       </c>
       <c r="B148" s="2" t="inlineStr">
@@ -7358,12 +7358,12 @@
       </c>
       <c r="C148" s="3" t="inlineStr">
         <is>
-          <t>Data Entry Specialist</t>
+          <t>Recepcion y facturacion de laboratorio clinico</t>
         </is>
       </c>
       <c r="D148" s="3" t="inlineStr">
         <is>
-          <t>ZEISS Group</t>
+          <t>Fundación Santa Fe de Bogotá</t>
         </is>
       </c>
       <c r="E148" s="7" t="n">
@@ -7375,13 +7375,13 @@
         </is>
       </c>
       <c r="G148" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/data-entry-specialist-at-zeiss-group-4467880077", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/recepcion-y-facturacion-de-laboratorio-clinico-1886760903", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H148" s="6" t="inlineStr"/>
       <c r="I148" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Auxiliar Administrativo / Asistente Virtual). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Alta coincidencia técnica en Herramientas Ofimáticas, Excel y Soporte Contable / Facturación. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J148" s="2" t="inlineStr">
@@ -7394,22 +7394,22 @@
     <row r="149" ht="22" customHeight="1">
       <c r="A149" s="2" t="inlineStr">
         <is>
-          <t>6051bd21daa83566</t>
+          <t>d45621f8599206ec</t>
         </is>
       </c>
       <c r="B149" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 18:38</t>
+          <t>2026-09-26 15:05</t>
         </is>
       </c>
       <c r="C149" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar contable y administrativo</t>
+          <t>Data Entry Specialist</t>
         </is>
       </c>
       <c r="D149" s="3" t="inlineStr">
         <is>
-          <t>distrigomez seguros</t>
+          <t>ZEISS Group</t>
         </is>
       </c>
       <c r="E149" s="7" t="n">
@@ -7421,14 +7421,10 @@
         </is>
       </c>
       <c r="G149" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-contable-y-administrativo-trabajo-desde-casa-en-pereira-3EEDFFC0D2447F8B61373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H149" s="6" t="inlineStr">
-        <is>
-          <t>$ 1.750.905,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/data-entry-specialist-at-zeiss-group-4467880077", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H149" s="6" t="inlineStr"/>
       <c r="I149" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Auxiliar Administrativo / Asistente Virtual). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -7444,7 +7440,7 @@
     <row r="150" ht="22" customHeight="1">
       <c r="A150" s="2" t="inlineStr">
         <is>
-          <t>1a7a81ed9e2a4160</t>
+          <t>6051bd21daa83566</t>
         </is>
       </c>
       <c r="B150" s="2" t="inlineStr">
@@ -7454,12 +7450,12 @@
       </c>
       <c r="C150" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar administrativo(a) - campus neiva</t>
+          <t>Auxiliar contable y administrativo</t>
         </is>
       </c>
       <c r="D150" s="3" t="inlineStr">
         <is>
-          <t>Universidad Cooperativa de Colombia</t>
+          <t>distrigomez seguros</t>
         </is>
       </c>
       <c r="E150" s="7" t="n">
@@ -7471,10 +7467,14 @@
         </is>
       </c>
       <c r="G150" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-administrativoa-campus-neiva-1886773020", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H150" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-contable-y-administrativo-trabajo-desde-casa-en-pereira-3EEDFFC0D2447F8B61373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H150" s="6" t="inlineStr">
+        <is>
+          <t>$ 1.750.905,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I150" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Auxiliar Administrativo / Asistente Virtual). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -7490,7 +7490,7 @@
     <row r="151" ht="22" customHeight="1">
       <c r="A151" s="2" t="inlineStr">
         <is>
-          <t>a81375d5a4201305</t>
+          <t>1a7a81ed9e2a4160</t>
         </is>
       </c>
       <c r="B151" s="2" t="inlineStr">
@@ -7500,12 +7500,12 @@
       </c>
       <c r="C151" s="3" t="inlineStr">
         <is>
-          <t>Digitador - bogotá</t>
+          <t>Auxiliar administrativo(a) - campus neiva</t>
         </is>
       </c>
       <c r="D151" s="3" t="inlineStr">
         <is>
-          <t>BUREAU VERITAS</t>
+          <t>Universidad Cooperativa de Colombia</t>
         </is>
       </c>
       <c r="E151" s="7" t="n">
@@ -7517,7 +7517,7 @@
         </is>
       </c>
       <c r="G151" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/digitador-bogota-1886762709", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-administrativoa-campus-neiva-1886773020", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H151" s="6" t="inlineStr"/>
@@ -7536,22 +7536,22 @@
     <row r="152" ht="22" customHeight="1">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t>9164fad20028594e</t>
+          <t>a81375d5a4201305</t>
         </is>
       </c>
       <c r="B152" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 17:03</t>
+          <t>2026-09-28 18:38</t>
         </is>
       </c>
       <c r="C152" s="3" t="inlineStr">
         <is>
-          <t>Digitador(a) de nómina</t>
+          <t>Digitador - bogotá</t>
         </is>
       </c>
       <c r="D152" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>BUREAU VERITAS</t>
         </is>
       </c>
       <c r="E152" s="7" t="n">
@@ -7563,7 +7563,7 @@
         </is>
       </c>
       <c r="G152" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/digitadora-de-nomina-1886773344", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/digitador-bogota-1886762709", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H152" s="6" t="inlineStr"/>
@@ -7582,7 +7582,7 @@
     <row r="153" ht="22" customHeight="1">
       <c r="A153" s="2" t="inlineStr">
         <is>
-          <t>eb9248ba68f06027</t>
+          <t>9164fad20028594e</t>
         </is>
       </c>
       <c r="B153" s="2" t="inlineStr">
@@ -7592,12 +7592,12 @@
       </c>
       <c r="C153" s="3" t="inlineStr">
         <is>
-          <t>Young Professional – Data Entry - Remote Work</t>
+          <t>Digitador(a) de nómina</t>
         </is>
       </c>
       <c r="D153" s="3" t="inlineStr">
         <is>
-          <t>BairesDev</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E153" s="7" t="n">
@@ -7609,7 +7609,7 @@
         </is>
       </c>
       <c r="G153" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/young-professional-%E2%80%93-data-entry-remote-work-at-bairesdev-4471917951", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/digitadora-de-nomina-1886773344", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H153" s="6" t="inlineStr"/>
@@ -7628,22 +7628,22 @@
     <row r="154" ht="22" customHeight="1">
       <c r="A154" s="2" t="inlineStr">
         <is>
-          <t>ab0015399fb0fd5a</t>
+          <t>eb9248ba68f06027</t>
         </is>
       </c>
       <c r="B154" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 16:51</t>
+          <t>2026-09-29 17:03</t>
         </is>
       </c>
       <c r="C154" s="3" t="inlineStr">
         <is>
-          <t>Cali- asistente administrativo y contable</t>
+          <t>Young Professional – Data Entry - Remote Work</t>
         </is>
       </c>
       <c r="D154" s="3" t="inlineStr">
         <is>
-          <t>GERENCIA SELECTA SAS</t>
+          <t>BairesDev</t>
         </is>
       </c>
       <c r="E154" s="7" t="n">
@@ -7655,7 +7655,7 @@
         </is>
       </c>
       <c r="G154" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/cali-asistente-administrativo-y-contable-1886774199", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/young-professional-%E2%80%93-data-entry-remote-work-at-bairesdev-4471917951", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H154" s="6" t="inlineStr"/>
@@ -7674,7 +7674,7 @@
     <row r="155" ht="22" customHeight="1">
       <c r="A155" s="2" t="inlineStr">
         <is>
-          <t>f151a5101fd2098d</t>
+          <t>ab0015399fb0fd5a</t>
         </is>
       </c>
       <c r="B155" s="2" t="inlineStr">
@@ -7684,12 +7684,12 @@
       </c>
       <c r="C155" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar contable y administrativo 212747-148845</t>
+          <t>Cali- asistente administrativo y contable</t>
         </is>
       </c>
       <c r="D155" s="3" t="inlineStr">
         <is>
-          <t>AGENCIA DE EMPLEO Y FOMENTO EMPRESARIAL COMPENSAR</t>
+          <t>GERENCIA SELECTA SAS</t>
         </is>
       </c>
       <c r="E155" s="7" t="n">
@@ -7701,7 +7701,7 @@
         </is>
       </c>
       <c r="G155" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-contable-y-administrativo-212747148845-1886774053", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/cali-asistente-administrativo-y-contable-1886774199", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H155" s="6" t="inlineStr"/>
@@ -7720,7 +7720,7 @@
     <row r="156" ht="22" customHeight="1">
       <c r="A156" s="2" t="inlineStr">
         <is>
-          <t>2ad924abc5b01201</t>
+          <t>f151a5101fd2098d</t>
         </is>
       </c>
       <c r="B156" s="2" t="inlineStr">
@@ -7730,7 +7730,7 @@
       </c>
       <c r="C156" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar administrativa y contable- mosquera- 1626546205-1</t>
+          <t>Auxiliar contable y administrativo 212747-148845</t>
         </is>
       </c>
       <c r="D156" s="3" t="inlineStr">
@@ -7747,7 +7747,7 @@
         </is>
       </c>
       <c r="G156" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-administrativa-y-contable-mosquera-16265462051-1886773852", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-contable-y-administrativo-212747148845-1886774053", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H156" s="6" t="inlineStr"/>
@@ -7766,7 +7766,7 @@
     <row r="157" ht="22" customHeight="1">
       <c r="A157" s="2" t="inlineStr">
         <is>
-          <t>cb0d1367aba57052</t>
+          <t>2ad924abc5b01201</t>
         </is>
       </c>
       <c r="B157" s="2" t="inlineStr">
@@ -7776,12 +7776,12 @@
       </c>
       <c r="C157" s="3" t="inlineStr">
         <is>
-          <t>Client Intake and Data Entry Specialist</t>
+          <t>Auxiliar administrativa y contable- mosquera- 1626546205-1</t>
         </is>
       </c>
       <c r="D157" s="3" t="inlineStr">
         <is>
-          <t>Job Duck</t>
+          <t>AGENCIA DE EMPLEO Y FOMENTO EMPRESARIAL COMPENSAR</t>
         </is>
       </c>
       <c r="E157" s="7" t="n">
@@ -7793,7 +7793,7 @@
         </is>
       </c>
       <c r="G157" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/client-intake-and-data-entry-specialist-at-job-duck-4473785617", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-administrativa-y-contable-mosquera-16265462051-1886773852", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H157" s="6" t="inlineStr"/>
@@ -7812,7 +7812,7 @@
     <row r="158" ht="22" customHeight="1">
       <c r="A158" s="2" t="inlineStr">
         <is>
-          <t>aa2ff4b012a2356b</t>
+          <t>cb0d1367aba57052</t>
         </is>
       </c>
       <c r="B158" s="2" t="inlineStr">
@@ -7822,12 +7822,12 @@
       </c>
       <c r="C158" s="3" t="inlineStr">
         <is>
-          <t>Data entry specialist</t>
+          <t>Client Intake and Data Entry Specialist</t>
         </is>
       </c>
       <c r="D158" s="3" t="inlineStr">
         <is>
-          <t>Naur Talent</t>
+          <t>Job Duck</t>
         </is>
       </c>
       <c r="E158" s="7" t="n">
@@ -7839,7 +7839,7 @@
         </is>
       </c>
       <c r="G158" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/data-entry-specialist-at-naur-talent-4473907227", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/client-intake-and-data-entry-specialist-at-job-duck-4473785617", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H158" s="6" t="inlineStr"/>
@@ -7858,22 +7858,22 @@
     <row r="159" ht="22" customHeight="1">
       <c r="A159" s="2" t="inlineStr">
         <is>
-          <t>0fb7813f6ca58c19</t>
+          <t>aa2ff4b012a2356b</t>
         </is>
       </c>
       <c r="B159" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 17:28</t>
+          <t>2026-09-30 16:51</t>
         </is>
       </c>
       <c r="C159" s="3" t="inlineStr">
         <is>
-          <t>Data Entry Assistant</t>
+          <t>Data entry specialist</t>
         </is>
       </c>
       <c r="D159" s="3" t="inlineStr">
         <is>
-          <t>NEO - New Estate Only</t>
+          <t>Naur Talent</t>
         </is>
       </c>
       <c r="E159" s="7" t="n">
@@ -7885,7 +7885,7 @@
         </is>
       </c>
       <c r="G159" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/data-entry-assistant-at-neo-new-estate-only-4474342064", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/data-entry-specialist-at-naur-talent-4473907227", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H159" s="6" t="inlineStr"/>
@@ -7904,22 +7904,22 @@
     <row r="160" ht="22" customHeight="1">
       <c r="A160" s="2" t="inlineStr">
         <is>
-          <t>e03aa4c6959d3eb4</t>
+          <t>0fb7813f6ca58c19</t>
         </is>
       </c>
       <c r="B160" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03 15:14</t>
+          <t>2026-10-01 17:28</t>
         </is>
       </c>
       <c r="C160" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar administrativo/a Vacante Inclusiva para personas con Discapacidad</t>
+          <t>Data Entry Assistant</t>
         </is>
       </c>
       <c r="D160" s="3" t="inlineStr">
         <is>
-          <t>CENTRO DE EMPLEO Y TALENTO COLSUBSIDIO</t>
+          <t>NEO - New Estate Only</t>
         </is>
       </c>
       <c r="E160" s="7" t="n">
@@ -7931,14 +7931,10 @@
         </is>
       </c>
       <c r="G160" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-administrativoa-vacante-inclusiva-para-personas-con-discapacidad-en-bogota-dc-C48470AF94C2CBCC61373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H160" s="6" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/data-entry-assistant-at-neo-new-estate-only-4474342064", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H160" s="6" t="inlineStr"/>
       <c r="I160" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Auxiliar Administrativo / Asistente Virtual). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -7954,7 +7950,7 @@
     <row r="161" ht="22" customHeight="1">
       <c r="A161" s="2" t="inlineStr">
         <is>
-          <t>1a638820869677f4</t>
+          <t>e03aa4c6959d3eb4</t>
         </is>
       </c>
       <c r="B161" s="2" t="inlineStr">
@@ -7964,12 +7960,12 @@
       </c>
       <c r="C161" s="3" t="inlineStr">
         <is>
-          <t>Asistente administrativa</t>
+          <t>Auxiliar administrativo/a Vacante Inclusiva para personas con Discapacidad</t>
         </is>
       </c>
       <c r="D161" s="3" t="inlineStr">
         <is>
-          <t>Valgroup Realty LLC</t>
+          <t>CENTRO DE EMPLEO Y TALENTO COLSUBSIDIO</t>
         </is>
       </c>
       <c r="E161" s="7" t="n">
@@ -7981,7 +7977,7 @@
         </is>
       </c>
       <c r="G161" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-asistente-administrativa-con-conocimiento-del-idioma-ingles-en-bucaramanga-E109D498CC2B20FD61373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-administrativoa-vacante-inclusiva-para-personas-con-discapacidad-en-bogota-dc-C48470AF94C2CBCC61373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H161" s="6" t="inlineStr">
@@ -8004,26 +8000,26 @@
     <row r="162" ht="22" customHeight="1">
       <c r="A162" s="2" t="inlineStr">
         <is>
-          <t>bab8c57875b70054</t>
+          <t>1a638820869677f4</t>
         </is>
       </c>
       <c r="B162" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 16:07</t>
+          <t>2026-10-03 15:14</t>
         </is>
       </c>
       <c r="C162" s="3" t="inlineStr">
         <is>
-          <t>Analista de Servicio al Cliente Digital / Personal con Discapacidad</t>
+          <t>Asistente administrativa</t>
         </is>
       </c>
       <c r="D162" s="3" t="inlineStr">
         <is>
-          <t>HOME BURGERS</t>
+          <t>Valgroup Realty LLC</t>
         </is>
       </c>
       <c r="E162" s="7" t="n">
-        <v>0.53</v>
+        <v>0.58</v>
       </c>
       <c r="F162" s="2" t="inlineStr">
         <is>
@@ -8031,17 +8027,17 @@
         </is>
       </c>
       <c r="G162" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-analista-de-servicio-al-cliente-digital-personal-con-discapacidad-en-bogota-dc-11CE94961396D4CF61373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-asistente-administrativa-con-conocimiento-del-idioma-ingles-en-bucaramanga-E109D498CC2B20FD61373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H162" s="6" t="inlineStr">
         <is>
-          <t>$ 1.750.000,00 (Mensual)</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="I162" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Auxiliar Administrativo / Asistente Virtual). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Auxiliar Administrativo / Asistente Virtual). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J162" s="2" t="inlineStr">
@@ -8054,7 +8050,7 @@
     <row r="163" ht="22" customHeight="1">
       <c r="A163" s="2" t="inlineStr">
         <is>
-          <t>e4553a32da3edf6d</t>
+          <t>bab8c57875b70054</t>
         </is>
       </c>
       <c r="B163" s="2" t="inlineStr">
@@ -8064,12 +8060,12 @@
       </c>
       <c r="C163" s="3" t="inlineStr">
         <is>
-          <t>Asesor de Servicio al Cliente / Remoto</t>
+          <t>Analista de Servicio al Cliente Digital / Personal con Discapacidad</t>
         </is>
       </c>
       <c r="D163" s="3" t="inlineStr">
         <is>
-          <t>SIIGO S.A.S</t>
+          <t>HOME BURGERS</t>
         </is>
       </c>
       <c r="E163" s="7" t="n">
@@ -8081,12 +8077,12 @@
         </is>
       </c>
       <c r="G163" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-asesor-de-servicio-al-cliente-remoto-en-bogota-dc-00C206C9966382F961373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-analista-de-servicio-al-cliente-digital-personal-con-discapacidad-en-bogota-dc-11CE94961396D4CF61373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H163" s="6" t="inlineStr">
         <is>
-          <t>$ 1.750.905,00 (Mensual)</t>
+          <t>$ 1.750.000,00 (Mensual)</t>
         </is>
       </c>
       <c r="I163" s="3" t="inlineStr">
@@ -8104,22 +8100,22 @@
     <row r="164" ht="22" customHeight="1">
       <c r="A164" s="2" t="inlineStr">
         <is>
-          <t>838f39602895a4e7</t>
+          <t>e4553a32da3edf6d</t>
         </is>
       </c>
       <c r="B164" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03 15:14</t>
+          <t>2026-09-24 16:07</t>
         </is>
       </c>
       <c r="C164" s="3" t="inlineStr">
         <is>
-          <t>Analista de facturación (billing analyst)/ inglés b2 /híbrido</t>
+          <t>Asesor de Servicio al Cliente / Remoto</t>
         </is>
       </c>
       <c r="D164" s="3" t="inlineStr">
         <is>
-          <t>MANPOWER</t>
+          <t>SIIGO S.A.S</t>
         </is>
       </c>
       <c r="E164" s="7" t="n">
@@ -8127,17 +8123,21 @@
       </c>
       <c r="F164" s="2" t="inlineStr">
         <is>
-          <t>Hibrido</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="G164" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-facturacion-billing-analyst-ingles-b2-hibrido-1886773841", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H164" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-asesor-de-servicio-al-cliente-remoto-en-bogota-dc-00C206C9966382F961373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H164" s="6" t="inlineStr">
+        <is>
+          <t>$ 1.750.905,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I164" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 53/100 - Afinidad Moderada] Alta coincidencia técnica en Herramientas Ofimáticas, Excel y Soporte Contable / Facturación. Modalidad: Modalidad híbrida / parcial. Alerta: Modalidad híbrida puede requerir presencia ocasional.</t>
+          <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Auxiliar Administrativo / Asistente Virtual). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J164" s="2" t="inlineStr">
@@ -8150,40 +8150,40 @@
     <row r="165" ht="22" customHeight="1">
       <c r="A165" s="2" t="inlineStr">
         <is>
-          <t>cd1036bcf66024dc</t>
+          <t>838f39602895a4e7</t>
         </is>
       </c>
       <c r="B165" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26 15:05</t>
+          <t>2026-10-03 15:14</t>
         </is>
       </c>
       <c r="C165" s="3" t="inlineStr">
         <is>
-          <t>Aprendiz practicante administrativo</t>
+          <t>Analista de facturación (billing analyst)/ inglés b2 /híbrido</t>
         </is>
       </c>
       <c r="D165" s="3" t="inlineStr">
         <is>
-          <t>Bold.co</t>
+          <t>MANPOWER</t>
         </is>
       </c>
       <c r="E165" s="7" t="n">
-        <v>0.5</v>
+        <v>0.53</v>
       </c>
       <c r="F165" s="2" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Hibrido</t>
         </is>
       </c>
       <c r="G165" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/aprendiz-practicante-administrativo-etapa-productiva-at-bold-4457032181", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-facturacion-billing-analyst-ingles-b2-hibrido-1886773841", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H165" s="6" t="inlineStr"/>
       <c r="I165" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Auxiliar Administrativo / Asistente Virtual). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 53/100 - Afinidad Moderada] Alta coincidencia técnica en Herramientas Ofimáticas, Excel y Soporte Contable / Facturación. Modalidad: Modalidad híbrida / parcial. Alerta: Modalidad híbrida puede requerir presencia ocasional.</t>
         </is>
       </c>
       <c r="J165" s="2" t="inlineStr">
@@ -8196,22 +8196,22 @@
     <row r="166" ht="22" customHeight="1">
       <c r="A166" s="2" t="inlineStr">
         <is>
-          <t>dbdce1eb16060a6a</t>
+          <t>cd1036bcf66024dc</t>
         </is>
       </c>
       <c r="B166" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 18:38</t>
+          <t>2026-09-26 15:05</t>
         </is>
       </c>
       <c r="C166" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar contable jr</t>
+          <t>Aprendiz practicante administrativo</t>
         </is>
       </c>
       <c r="D166" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Bold.co</t>
         </is>
       </c>
       <c r="E166" s="7" t="n">
@@ -8223,7 +8223,7 @@
         </is>
       </c>
       <c r="G166" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-contable-jr-1886767584", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/aprendiz-practicante-administrativo-etapa-productiva-at-bold-4457032181", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H166" s="6" t="inlineStr"/>
@@ -8242,7 +8242,7 @@
     <row r="167" ht="22" customHeight="1">
       <c r="A167" s="2" t="inlineStr">
         <is>
-          <t>550ad8afea6faf9b</t>
+          <t>dbdce1eb16060a6a</t>
         </is>
       </c>
       <c r="B167" s="2" t="inlineStr">
@@ -8252,12 +8252,12 @@
       </c>
       <c r="C167" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar Contable Junior</t>
+          <t>Auxiliar contable jr</t>
         </is>
       </c>
       <c r="D167" s="3" t="inlineStr">
         <is>
-          <t>Ariadna Communications Group</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E167" s="7" t="n">
@@ -8269,7 +8269,7 @@
         </is>
       </c>
       <c r="G167" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/auxiliar-contable-junior-at-ariadna-communications-group-4472764062", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-contable-jr-1886767584", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H167" s="6" t="inlineStr"/>
@@ -8284,6 +8284,52 @@
         </is>
       </c>
       <c r="K167" s="3" t="inlineStr"/>
+    </row>
+    <row r="168" ht="22" customHeight="1">
+      <c r="A168" s="2" t="inlineStr">
+        <is>
+          <t>550ad8afea6faf9b</t>
+        </is>
+      </c>
+      <c r="B168" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28 18:38</t>
+        </is>
+      </c>
+      <c r="C168" s="3" t="inlineStr">
+        <is>
+          <t>Auxiliar Contable Junior</t>
+        </is>
+      </c>
+      <c r="D168" s="3" t="inlineStr">
+        <is>
+          <t>Ariadna Communications Group</t>
+        </is>
+      </c>
+      <c r="E168" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F168" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G168" s="5">
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/auxiliar-contable-junior-at-ariadna-communications-group-4472764062", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H168" s="6" t="inlineStr"/>
+      <c r="I168" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Auxiliar Administrativo / Asistente Virtual). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J168" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K168" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
chore(tracker): actualizacion diaria de vacantes 2026-10-31
</commit_message>
<xml_diff>
--- a/output/profile_6_auxiliar_administrativo_tracker.xlsx
+++ b/output/profile_6_auxiliar_administrativo_tracker.xlsx
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K252"/>
+  <dimension ref="A1:K253"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -11528,26 +11528,26 @@
     <row r="238" ht="22" customHeight="1">
       <c r="A238" s="2" t="inlineStr">
         <is>
-          <t>bab8c57875b70054</t>
+          <t>09c45520a20e80b8</t>
         </is>
       </c>
       <c r="B238" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 16:07</t>
+          <t>2026-10-31 16:09</t>
         </is>
       </c>
       <c r="C238" s="3" t="inlineStr">
         <is>
-          <t>Analista de Servicio al Cliente Digital / Personal con Discapacidad</t>
+          <t>Digitador(a) de nómina</t>
         </is>
       </c>
       <c r="D238" s="3" t="inlineStr">
         <is>
-          <t>HOME BURGERS</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E238" s="7" t="n">
-        <v>0.53</v>
+        <v>0.58</v>
       </c>
       <c r="F238" s="2" t="inlineStr">
         <is>
@@ -11555,17 +11555,13 @@
         </is>
       </c>
       <c r="G238" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-analista-de-servicio-al-cliente-digital-personal-con-discapacidad-en-bogota-dc-11CE94961396D4CF61373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H238" s="6" t="inlineStr">
-        <is>
-          <t>$ 1.750.000,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/digitadora-de-nomina-1886787772", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H238" s="6" t="inlineStr"/>
       <c r="I238" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Auxiliar Administrativo / Asistente Virtual). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Auxiliar Administrativo / Asistente Virtual). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J238" s="2" t="inlineStr">
@@ -11578,7 +11574,7 @@
     <row r="239" ht="22" customHeight="1">
       <c r="A239" s="2" t="inlineStr">
         <is>
-          <t>e4553a32da3edf6d</t>
+          <t>bab8c57875b70054</t>
         </is>
       </c>
       <c r="B239" s="2" t="inlineStr">
@@ -11588,12 +11584,12 @@
       </c>
       <c r="C239" s="3" t="inlineStr">
         <is>
-          <t>Asesor de Servicio al Cliente / Remoto</t>
+          <t>Analista de Servicio al Cliente Digital / Personal con Discapacidad</t>
         </is>
       </c>
       <c r="D239" s="3" t="inlineStr">
         <is>
-          <t>SIIGO S.A.S</t>
+          <t>HOME BURGERS</t>
         </is>
       </c>
       <c r="E239" s="7" t="n">
@@ -11605,12 +11601,12 @@
         </is>
       </c>
       <c r="G239" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-asesor-de-servicio-al-cliente-remoto-en-bogota-dc-00C206C9966382F961373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-analista-de-servicio-al-cliente-digital-personal-con-discapacidad-en-bogota-dc-11CE94961396D4CF61373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H239" s="6" t="inlineStr">
         <is>
-          <t>$ 1.750.905,00 (Mensual)</t>
+          <t>$ 1.750.000,00 (Mensual)</t>
         </is>
       </c>
       <c r="I239" s="3" t="inlineStr">
@@ -11628,22 +11624,22 @@
     <row r="240" ht="22" customHeight="1">
       <c r="A240" s="2" t="inlineStr">
         <is>
-          <t>838f39602895a4e7</t>
+          <t>e4553a32da3edf6d</t>
         </is>
       </c>
       <c r="B240" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03 15:14</t>
+          <t>2026-09-24 16:07</t>
         </is>
       </c>
       <c r="C240" s="3" t="inlineStr">
         <is>
-          <t>Analista de facturación (billing analyst)/ inglés b2 /híbrido</t>
+          <t>Asesor de Servicio al Cliente / Remoto</t>
         </is>
       </c>
       <c r="D240" s="3" t="inlineStr">
         <is>
-          <t>MANPOWER</t>
+          <t>SIIGO S.A.S</t>
         </is>
       </c>
       <c r="E240" s="7" t="n">
@@ -11651,17 +11647,21 @@
       </c>
       <c r="F240" s="2" t="inlineStr">
         <is>
-          <t>Hibrido</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="G240" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-facturacion-billing-analyst-ingles-b2-hibrido-1886773841", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H240" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-asesor-de-servicio-al-cliente-remoto-en-bogota-dc-00C206C9966382F961373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H240" s="6" t="inlineStr">
+        <is>
+          <t>$ 1.750.905,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I240" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 53/100 - Afinidad Moderada] Alta coincidencia técnica en Herramientas Ofimáticas, Excel y Soporte Contable / Facturación. Modalidad: Modalidad híbrida / parcial. Alerta: Modalidad híbrida puede requerir presencia ocasional.</t>
+          <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Auxiliar Administrativo / Asistente Virtual). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J240" s="2" t="inlineStr">
@@ -11674,22 +11674,22 @@
     <row r="241" ht="22" customHeight="1">
       <c r="A241" s="2" t="inlineStr">
         <is>
-          <t>c2dea1f07ef53647</t>
+          <t>838f39602895a4e7</t>
         </is>
       </c>
       <c r="B241" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06 17:14</t>
+          <t>2026-10-03 15:14</t>
         </is>
       </c>
       <c r="C241" s="3" t="inlineStr">
         <is>
-          <t>Consultor sap fi-gl / fi-aa s/4hana - remoto colombia</t>
+          <t>Analista de facturación (billing analyst)/ inglés b2 /híbrido</t>
         </is>
       </c>
       <c r="D241" s="3" t="inlineStr">
         <is>
-          <t>TALYCAP GLOBAL SAS</t>
+          <t>MANPOWER</t>
         </is>
       </c>
       <c r="E241" s="7" t="n">
@@ -11697,17 +11697,17 @@
       </c>
       <c r="F241" s="2" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Hibrido</t>
         </is>
       </c>
       <c r="G241" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/consultor-sap-figl-fiaa-s-4hana-remoto-colombia-1886776900", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-facturacion-billing-analyst-ingles-b2-hibrido-1886773841", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H241" s="6" t="inlineStr"/>
       <c r="I241" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Auxiliar Administrativo / Asistente Virtual). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 53/100 - Afinidad Moderada] Alta coincidencia técnica en Herramientas Ofimáticas, Excel y Soporte Contable / Facturación. Modalidad: Modalidad híbrida / parcial. Alerta: Modalidad híbrida puede requerir presencia ocasional.</t>
         </is>
       </c>
       <c r="J241" s="2" t="inlineStr">
@@ -11720,22 +11720,22 @@
     <row r="242" ht="22" customHeight="1">
       <c r="A242" s="2" t="inlineStr">
         <is>
-          <t>d55c5bcc13a598dc</t>
+          <t>c2dea1f07ef53647</t>
         </is>
       </c>
       <c r="B242" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07 17:52</t>
+          <t>2026-10-06 17:14</t>
         </is>
       </c>
       <c r="C242" s="3" t="inlineStr">
         <is>
-          <t>Asesor(a) de servicio al cliente bilingüe</t>
+          <t>Consultor sap fi-gl / fi-aa s/4hana - remoto colombia</t>
         </is>
       </c>
       <c r="D242" s="3" t="inlineStr">
         <is>
-          <t>Empresa en expansión</t>
+          <t>TALYCAP GLOBAL SAS</t>
         </is>
       </c>
       <c r="E242" s="7" t="n">
@@ -11747,14 +11747,10 @@
         </is>
       </c>
       <c r="G242" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-asesora-de-servicio-al-cliente-bilingue-home-office-ingles-c1-con-experiencia-en-estados-unidos-D522AAAB4F954B8061373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H242" s="6" t="inlineStr">
-        <is>
-          <t>$ 3.500.000,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/consultor-sap-figl-fiaa-s-4hana-remoto-colombia-1886776900", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H242" s="6" t="inlineStr"/>
       <c r="I242" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Auxiliar Administrativo / Asistente Virtual). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -11770,22 +11766,22 @@
     <row r="243" ht="22" customHeight="1">
       <c r="A243" s="2" t="inlineStr">
         <is>
-          <t>08504d61be6d0f7f</t>
+          <t>d55c5bcc13a598dc</t>
         </is>
       </c>
       <c r="B243" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14 15:54</t>
+          <t>2026-10-07 17:52</t>
         </is>
       </c>
       <c r="C243" s="3" t="inlineStr">
         <is>
-          <t>Consultor sap datasphere - remoto</t>
+          <t>Asesor(a) de servicio al cliente bilingüe</t>
         </is>
       </c>
       <c r="D243" s="3" t="inlineStr">
         <is>
-          <t>Cinte Colombia SAS</t>
+          <t>Empresa en expansión</t>
         </is>
       </c>
       <c r="E243" s="7" t="n">
@@ -11797,10 +11793,14 @@
         </is>
       </c>
       <c r="G243" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/consultor-sap-datasphere-remoto-1886759862", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H243" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-asesora-de-servicio-al-cliente-bilingue-home-office-ingles-c1-con-experiencia-en-estados-unidos-D522AAAB4F954B8061373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H243" s="6" t="inlineStr">
+        <is>
+          <t>$ 3.500.000,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I243" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Auxiliar Administrativo / Asistente Virtual). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -11816,22 +11816,22 @@
     <row r="244" ht="22" customHeight="1">
       <c r="A244" s="2" t="inlineStr">
         <is>
-          <t>fd0cf1451b259786</t>
+          <t>08504d61be6d0f7f</t>
         </is>
       </c>
       <c r="B244" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16 15:24</t>
+          <t>2026-10-14 15:54</t>
         </is>
       </c>
       <c r="C244" s="3" t="inlineStr">
         <is>
-          <t>Asesor de Servicio al Cliente / Remoto</t>
+          <t>Consultor sap datasphere - remoto</t>
         </is>
       </c>
       <c r="D244" s="3" t="inlineStr">
         <is>
-          <t>SIIGO S.A.S</t>
+          <t>Cinte Colombia SAS</t>
         </is>
       </c>
       <c r="E244" s="7" t="n">
@@ -11843,14 +11843,10 @@
         </is>
       </c>
       <c r="G244" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-asesor-de-servicio-al-cliente-remoto-en-bogota-dc-0757873A03E0E43661373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H244" s="6" t="inlineStr">
-        <is>
-          <t>$ 1.750.905,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/consultor-sap-datasphere-remoto-1886759862", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H244" s="6" t="inlineStr"/>
       <c r="I244" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Auxiliar Administrativo / Asistente Virtual). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -11866,22 +11862,22 @@
     <row r="245" ht="22" customHeight="1">
       <c r="A245" s="2" t="inlineStr">
         <is>
-          <t>f4f5539b99aa321c</t>
+          <t>fd0cf1451b259786</t>
         </is>
       </c>
       <c r="B245" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17 14:17</t>
+          <t>2026-10-16 15:24</t>
         </is>
       </c>
       <c r="C245" s="3" t="inlineStr">
         <is>
-          <t>Analista de cartera y servicio al cliente</t>
+          <t>Asesor de Servicio al Cliente / Remoto</t>
         </is>
       </c>
       <c r="D245" s="3" t="inlineStr">
         <is>
-          <t>AMANECER MEDICO SAS</t>
+          <t>SIIGO S.A.S</t>
         </is>
       </c>
       <c r="E245" s="7" t="n">
@@ -11893,10 +11889,14 @@
         </is>
       </c>
       <c r="G245" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/analista-de-cartera-y-servicio-al-cliente-at-amanecer-medico-sas-4480538113", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H245" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-asesor-de-servicio-al-cliente-remoto-en-bogota-dc-0757873A03E0E43661373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H245" s="6" t="inlineStr">
+        <is>
+          <t>$ 1.750.905,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I245" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Auxiliar Administrativo / Asistente Virtual). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -11912,22 +11912,22 @@
     <row r="246" ht="22" customHeight="1">
       <c r="A246" s="2" t="inlineStr">
         <is>
-          <t>5f6b837cd82a3734</t>
+          <t>f4f5539b99aa321c</t>
         </is>
       </c>
       <c r="B246" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:31</t>
+          <t>2026-10-17 14:17</t>
         </is>
       </c>
       <c r="C246" s="3" t="inlineStr">
         <is>
-          <t>Asesor de Servicio al Cliente Trilingüe Ingles B1 , Frances B2</t>
+          <t>Analista de cartera y servicio al cliente</t>
         </is>
       </c>
       <c r="D246" s="3" t="inlineStr">
         <is>
-          <t>Gi Group Colombia</t>
+          <t>AMANECER MEDICO SAS</t>
         </is>
       </c>
       <c r="E246" s="7" t="n">
@@ -11939,14 +11939,10 @@
         </is>
       </c>
       <c r="G246" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-asesor-de-servicio-al-cliente-trilingue-ingles-b1-frances-b2-en-bogota-dc-578A57277B8BC58561373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H246" s="6" t="inlineStr">
-        <is>
-          <t>$ 3.061.000,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/analista-de-cartera-y-servicio-al-cliente-at-amanecer-medico-sas-4480538113", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H246" s="6" t="inlineStr"/>
       <c r="I246" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Auxiliar Administrativo / Asistente Virtual). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -11962,26 +11958,26 @@
     <row r="247" ht="22" customHeight="1">
       <c r="A247" s="2" t="inlineStr">
         <is>
-          <t>cd1036bcf66024dc</t>
+          <t>5f6b837cd82a3734</t>
         </is>
       </c>
       <c r="B247" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26 15:05</t>
+          <t>2026-10-29 17:31</t>
         </is>
       </c>
       <c r="C247" s="3" t="inlineStr">
         <is>
-          <t>Aprendiz practicante administrativo</t>
+          <t>Asesor de Servicio al Cliente Trilingüe Ingles B1 , Frances B2</t>
         </is>
       </c>
       <c r="D247" s="3" t="inlineStr">
         <is>
-          <t>Bold.co</t>
+          <t>Gi Group Colombia</t>
         </is>
       </c>
       <c r="E247" s="7" t="n">
-        <v>0.5</v>
+        <v>0.53</v>
       </c>
       <c r="F247" s="2" t="inlineStr">
         <is>
@@ -11989,13 +11985,17 @@
         </is>
       </c>
       <c r="G247" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/aprendiz-practicante-administrativo-etapa-productiva-at-bold-4457032181", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H247" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-asesor-de-servicio-al-cliente-trilingue-ingles-b1-frances-b2-en-bogota-dc-578A57277B8BC58561373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H247" s="6" t="inlineStr">
+        <is>
+          <t>$ 3.061.000,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I247" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Auxiliar Administrativo / Asistente Virtual). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Auxiliar Administrativo / Asistente Virtual). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J247" s="2" t="inlineStr">
@@ -12008,22 +12008,22 @@
     <row r="248" ht="22" customHeight="1">
       <c r="A248" s="2" t="inlineStr">
         <is>
-          <t>dbdce1eb16060a6a</t>
+          <t>cd1036bcf66024dc</t>
         </is>
       </c>
       <c r="B248" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 18:38</t>
+          <t>2026-09-26 15:05</t>
         </is>
       </c>
       <c r="C248" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar contable jr</t>
+          <t>Aprendiz practicante administrativo</t>
         </is>
       </c>
       <c r="D248" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Bold.co</t>
         </is>
       </c>
       <c r="E248" s="7" t="n">
@@ -12035,7 +12035,7 @@
         </is>
       </c>
       <c r="G248" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-contable-jr-1886767584", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/aprendiz-practicante-administrativo-etapa-productiva-at-bold-4457032181", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H248" s="6" t="inlineStr"/>
@@ -12054,7 +12054,7 @@
     <row r="249" ht="22" customHeight="1">
       <c r="A249" s="2" t="inlineStr">
         <is>
-          <t>550ad8afea6faf9b</t>
+          <t>dbdce1eb16060a6a</t>
         </is>
       </c>
       <c r="B249" s="2" t="inlineStr">
@@ -12064,12 +12064,12 @@
       </c>
       <c r="C249" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar Contable Junior</t>
+          <t>Auxiliar contable jr</t>
         </is>
       </c>
       <c r="D249" s="3" t="inlineStr">
         <is>
-          <t>Ariadna Communications Group</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E249" s="7" t="n">
@@ -12081,7 +12081,7 @@
         </is>
       </c>
       <c r="G249" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/auxiliar-contable-junior-at-ariadna-communications-group-4472764062", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-contable-jr-1886767584", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H249" s="6" t="inlineStr"/>
@@ -12100,12 +12100,12 @@
     <row r="250" ht="22" customHeight="1">
       <c r="A250" s="2" t="inlineStr">
         <is>
-          <t>e8956f3876a2127b</t>
+          <t>550ad8afea6faf9b</t>
         </is>
       </c>
       <c r="B250" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15 15:43</t>
+          <t>2026-09-28 18:38</t>
         </is>
       </c>
       <c r="C250" s="3" t="inlineStr">
@@ -12115,7 +12115,7 @@
       </c>
       <c r="D250" s="3" t="inlineStr">
         <is>
-          <t>Empresa Privada</t>
+          <t>Ariadna Communications Group</t>
         </is>
       </c>
       <c r="E250" s="7" t="n">
@@ -12127,7 +12127,7 @@
         </is>
       </c>
       <c r="G250" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/auxiliar-contable-junior-at-private-company-4479719285", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/auxiliar-contable-junior-at-ariadna-communications-group-4472764062", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H250" s="6" t="inlineStr"/>
@@ -12146,22 +12146,22 @@
     <row r="251" ht="22" customHeight="1">
       <c r="A251" s="2" t="inlineStr">
         <is>
-          <t>1882fc6c9f917501</t>
+          <t>e8956f3876a2127b</t>
         </is>
       </c>
       <c r="B251" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27 16:24</t>
+          <t>2026-10-15 15:43</t>
         </is>
       </c>
       <c r="C251" s="3" t="inlineStr">
         <is>
-          <t>Representante de casino virtual / presentadora junior - sin experiencia</t>
+          <t>Auxiliar Contable Junior</t>
         </is>
       </c>
       <c r="D251" s="3" t="inlineStr">
         <is>
-          <t>INTEGRITY STAFFING SOLUTIONS COLOMBIA SAS</t>
+          <t>Empresa Privada</t>
         </is>
       </c>
       <c r="E251" s="7" t="n">
@@ -12173,7 +12173,7 @@
         </is>
       </c>
       <c r="G251" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/representante-de-casino-virtual-presentadora-junior-sin-experiencia-1886785447", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/auxiliar-contable-junior-at-private-company-4479719285", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H251" s="6" t="inlineStr"/>
@@ -12192,22 +12192,22 @@
     <row r="252" ht="22" customHeight="1">
       <c r="A252" s="2" t="inlineStr">
         <is>
-          <t>cab18ea45983ae06</t>
+          <t>1882fc6c9f917501</t>
         </is>
       </c>
       <c r="B252" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:08</t>
+          <t>2026-10-27 16:24</t>
         </is>
       </c>
       <c r="C252" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar Contable Junior</t>
+          <t>Representante de casino virtual / presentadora junior - sin experiencia</t>
         </is>
       </c>
       <c r="D252" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>INTEGRITY STAFFING SOLUTIONS COLOMBIA SAS</t>
         </is>
       </c>
       <c r="E252" s="7" t="n">
@@ -12219,7 +12219,7 @@
         </is>
       </c>
       <c r="G252" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/auxiliar-contable-junior-at-empresa-confidencial-4485227901", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/representante-de-casino-virtual-presentadora-junior-sin-experiencia-1886785447", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H252" s="6" t="inlineStr"/>
@@ -12234,6 +12234,52 @@
         </is>
       </c>
       <c r="K252" s="3" t="inlineStr"/>
+    </row>
+    <row r="253" ht="22" customHeight="1">
+      <c r="A253" s="2" t="inlineStr">
+        <is>
+          <t>cab18ea45983ae06</t>
+        </is>
+      </c>
+      <c r="B253" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 17:08</t>
+        </is>
+      </c>
+      <c r="C253" s="3" t="inlineStr">
+        <is>
+          <t>Auxiliar Contable Junior</t>
+        </is>
+      </c>
+      <c r="D253" s="3" t="inlineStr">
+        <is>
+          <t>Confidencial</t>
+        </is>
+      </c>
+      <c r="E253" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F253" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G253" s="5">
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/auxiliar-contable-junior-at-empresa-confidencial-4485227901", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H253" s="6" t="inlineStr"/>
+      <c r="I253" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Auxiliar Administrativo / Asistente Virtual). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J253" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K253" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>